<commit_message>
Case2 revalidated with the final code
</commit_message>
<xml_diff>
--- a/01_Validasyon/Case2/case2Validasyon.xlsx
+++ b/01_Validasyon/Case2/case2Validasyon.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\barankucukcay\Desktop\Ablation-Modeling\01_Validasyon\Case2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2623AD27-6012-4FA2-8D8D-43E43EA275B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{443596FA-6E32-4836-BF2B-BBBED481B9BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1363,892 +1363,892 @@
                   <c:v>200000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>199494</c:v>
+                  <c:v>199489</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>198977</c:v>
+                  <c:v>198971</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>198456</c:v>
+                  <c:v>198449</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>197933</c:v>
+                  <c:v>197926</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>197409</c:v>
+                  <c:v>197402</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>196884</c:v>
+                  <c:v>196877</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>196357</c:v>
+                  <c:v>196350</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>195830</c:v>
+                  <c:v>195822</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>195301</c:v>
+                  <c:v>195293</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>194771</c:v>
+                  <c:v>194763</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>194239</c:v>
+                  <c:v>194231</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>193707</c:v>
+                  <c:v>193698</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>193174</c:v>
+                  <c:v>193165</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>192639</c:v>
+                  <c:v>192630</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>192103</c:v>
+                  <c:v>192094</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>191566</c:v>
+                  <c:v>191557</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>191029</c:v>
+                  <c:v>191019</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>190490</c:v>
+                  <c:v>190480</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>189950</c:v>
+                  <c:v>189940</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>189409</c:v>
+                  <c:v>189398</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>188867</c:v>
+                  <c:v>188856</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>188325</c:v>
+                  <c:v>188314</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>187781</c:v>
+                  <c:v>187770</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>187237</c:v>
+                  <c:v>187225</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>186691</c:v>
+                  <c:v>186679</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>186145</c:v>
+                  <c:v>186133</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>185598</c:v>
+                  <c:v>185586</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>185050</c:v>
+                  <c:v>185037</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>184502</c:v>
+                  <c:v>184489</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>183952</c:v>
+                  <c:v>183939</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>183402</c:v>
+                  <c:v>183389</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>182851</c:v>
+                  <c:v>182838</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>182300</c:v>
+                  <c:v>182286</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>181748</c:v>
+                  <c:v>181734</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>181195</c:v>
+                  <c:v>181181</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>180642</c:v>
+                  <c:v>180627</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>180088</c:v>
+                  <c:v>180073</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>179534</c:v>
+                  <c:v>179519</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>178979</c:v>
+                  <c:v>178964</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>178424</c:v>
+                  <c:v>178408</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>177868</c:v>
+                  <c:v>177852</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>177312</c:v>
+                  <c:v>177296</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>176756</c:v>
+                  <c:v>176739</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>176199</c:v>
+                  <c:v>176182</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>175642</c:v>
+                  <c:v>175625</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>175084</c:v>
+                  <c:v>175067</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>174527</c:v>
+                  <c:v>174509</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>173969</c:v>
+                  <c:v>173951</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>173410</c:v>
+                  <c:v>173392</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>172852</c:v>
+                  <c:v>172834</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>172294</c:v>
+                  <c:v>172275</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>171735</c:v>
+                  <c:v>171716</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>171176</c:v>
+                  <c:v>171157</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>170618</c:v>
+                  <c:v>170598</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>170059</c:v>
+                  <c:v>170039</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>169501</c:v>
+                  <c:v>169480</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>168942</c:v>
+                  <c:v>168921</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>168384</c:v>
+                  <c:v>168363</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>167825</c:v>
+                  <c:v>167804</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>167267</c:v>
+                  <c:v>167246</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>166709</c:v>
+                  <c:v>166688</c:v>
                 </c:pt>
                 <c:pt idx="62">
-                  <c:v>166151</c:v>
+                  <c:v>166130</c:v>
                 </c:pt>
                 <c:pt idx="63">
-                  <c:v>165594</c:v>
+                  <c:v>165572</c:v>
                 </c:pt>
                 <c:pt idx="64">
-                  <c:v>165037</c:v>
+                  <c:v>165015</c:v>
                 </c:pt>
                 <c:pt idx="65">
-                  <c:v>164480</c:v>
+                  <c:v>164458</c:v>
                 </c:pt>
                 <c:pt idx="66">
-                  <c:v>163924</c:v>
+                  <c:v>163901</c:v>
                 </c:pt>
                 <c:pt idx="67">
-                  <c:v>163368</c:v>
+                  <c:v>163345</c:v>
                 </c:pt>
                 <c:pt idx="68">
-                  <c:v>162812</c:v>
+                  <c:v>162789</c:v>
                 </c:pt>
                 <c:pt idx="69">
-                  <c:v>162257</c:v>
+                  <c:v>162234</c:v>
                 </c:pt>
                 <c:pt idx="70">
-                  <c:v>161703</c:v>
+                  <c:v>161679</c:v>
                 </c:pt>
                 <c:pt idx="71">
-                  <c:v>161149</c:v>
+                  <c:v>161125</c:v>
                 </c:pt>
                 <c:pt idx="72">
-                  <c:v>160596</c:v>
+                  <c:v>160572</c:v>
                 </c:pt>
                 <c:pt idx="73">
-                  <c:v>160043</c:v>
+                  <c:v>160019</c:v>
                 </c:pt>
                 <c:pt idx="74">
-                  <c:v>159492</c:v>
+                  <c:v>159467</c:v>
                 </c:pt>
                 <c:pt idx="75">
-                  <c:v>158940</c:v>
+                  <c:v>158915</c:v>
                 </c:pt>
                 <c:pt idx="76">
-                  <c:v>158390</c:v>
+                  <c:v>158365</c:v>
                 </c:pt>
                 <c:pt idx="77">
-                  <c:v>157841</c:v>
+                  <c:v>157815</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v>157292</c:v>
+                  <c:v>157266</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v>156744</c:v>
+                  <c:v>156718</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v>156197</c:v>
+                  <c:v>156171</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>155652</c:v>
+                  <c:v>155625</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>155107</c:v>
+                  <c:v>155080</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>154563</c:v>
+                  <c:v>154536</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>154020</c:v>
+                  <c:v>153993</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v>153479</c:v>
+                  <c:v>153452</c:v>
                 </c:pt>
                 <c:pt idx="86">
-                  <c:v>152939</c:v>
+                  <c:v>152911</c:v>
                 </c:pt>
                 <c:pt idx="87">
-                  <c:v>152400</c:v>
+                  <c:v>152372</c:v>
                 </c:pt>
                 <c:pt idx="88">
-                  <c:v>151862</c:v>
+                  <c:v>151834</c:v>
                 </c:pt>
                 <c:pt idx="89">
-                  <c:v>151325</c:v>
+                  <c:v>151297</c:v>
                 </c:pt>
                 <c:pt idx="90">
-                  <c:v>150790</c:v>
+                  <c:v>150762</c:v>
                 </c:pt>
                 <c:pt idx="91">
-                  <c:v>150257</c:v>
+                  <c:v>150228</c:v>
                 </c:pt>
                 <c:pt idx="92">
-                  <c:v>149724</c:v>
+                  <c:v>149696</c:v>
                 </c:pt>
                 <c:pt idx="93">
-                  <c:v>149194</c:v>
+                  <c:v>149165</c:v>
                 </c:pt>
                 <c:pt idx="94">
-                  <c:v>148664</c:v>
+                  <c:v>148635</c:v>
                 </c:pt>
                 <c:pt idx="95">
-                  <c:v>148137</c:v>
+                  <c:v>148107</c:v>
                 </c:pt>
                 <c:pt idx="96">
-                  <c:v>147611</c:v>
+                  <c:v>147581</c:v>
                 </c:pt>
                 <c:pt idx="97">
-                  <c:v>147086</c:v>
+                  <c:v>147057</c:v>
                 </c:pt>
                 <c:pt idx="98">
-                  <c:v>146564</c:v>
+                  <c:v>146534</c:v>
                 </c:pt>
                 <c:pt idx="99">
-                  <c:v>146043</c:v>
+                  <c:v>146013</c:v>
                 </c:pt>
                 <c:pt idx="100">
-                  <c:v>145524</c:v>
+                  <c:v>145493</c:v>
                 </c:pt>
                 <c:pt idx="101">
-                  <c:v>145006</c:v>
+                  <c:v>144976</c:v>
                 </c:pt>
                 <c:pt idx="102">
-                  <c:v>144491</c:v>
+                  <c:v>144461</c:v>
                 </c:pt>
                 <c:pt idx="103">
-                  <c:v>143977</c:v>
+                  <c:v>143947</c:v>
                 </c:pt>
                 <c:pt idx="104">
-                  <c:v>143466</c:v>
+                  <c:v>143435</c:v>
                 </c:pt>
                 <c:pt idx="105">
-                  <c:v>142956</c:v>
+                  <c:v>142926</c:v>
                 </c:pt>
                 <c:pt idx="106">
-                  <c:v>142449</c:v>
+                  <c:v>142418</c:v>
                 </c:pt>
                 <c:pt idx="107">
-                  <c:v>141944</c:v>
+                  <c:v>141913</c:v>
                 </c:pt>
                 <c:pt idx="108">
-                  <c:v>141440</c:v>
+                  <c:v>141409</c:v>
                 </c:pt>
                 <c:pt idx="109">
-                  <c:v>140939</c:v>
+                  <c:v>140908</c:v>
                 </c:pt>
                 <c:pt idx="110">
-                  <c:v>140441</c:v>
+                  <c:v>140409</c:v>
                 </c:pt>
                 <c:pt idx="111">
-                  <c:v>139944</c:v>
+                  <c:v>139913</c:v>
                 </c:pt>
                 <c:pt idx="112">
-                  <c:v>139450</c:v>
+                  <c:v>139418</c:v>
                 </c:pt>
                 <c:pt idx="113">
-                  <c:v>138958</c:v>
+                  <c:v>138926</c:v>
                 </c:pt>
                 <c:pt idx="114">
-                  <c:v>138468</c:v>
+                  <c:v>138437</c:v>
                 </c:pt>
                 <c:pt idx="115">
-                  <c:v>137981</c:v>
+                  <c:v>137950</c:v>
                 </c:pt>
                 <c:pt idx="116">
-                  <c:v>137497</c:v>
+                  <c:v>137465</c:v>
                 </c:pt>
                 <c:pt idx="117">
-                  <c:v>137015</c:v>
+                  <c:v>136983</c:v>
                 </c:pt>
                 <c:pt idx="118">
-                  <c:v>136535</c:v>
+                  <c:v>136503</c:v>
                 </c:pt>
                 <c:pt idx="119">
-                  <c:v>136058</c:v>
+                  <c:v>136026</c:v>
                 </c:pt>
                 <c:pt idx="120">
-                  <c:v>135584</c:v>
+                  <c:v>135552</c:v>
                 </c:pt>
                 <c:pt idx="121">
-                  <c:v>135113</c:v>
+                  <c:v>135080</c:v>
                 </c:pt>
                 <c:pt idx="122">
-                  <c:v>134644</c:v>
+                  <c:v>134611</c:v>
                 </c:pt>
                 <c:pt idx="123">
-                  <c:v>134178</c:v>
+                  <c:v>134145</c:v>
                 </c:pt>
                 <c:pt idx="124">
-                  <c:v>133714</c:v>
+                  <c:v>133682</c:v>
                 </c:pt>
                 <c:pt idx="125">
-                  <c:v>133254</c:v>
+                  <c:v>133221</c:v>
                 </c:pt>
                 <c:pt idx="126">
-                  <c:v>132796</c:v>
+                  <c:v>132764</c:v>
                 </c:pt>
                 <c:pt idx="127">
-                  <c:v>132342</c:v>
+                  <c:v>132309</c:v>
                 </c:pt>
                 <c:pt idx="128">
-                  <c:v>131890</c:v>
+                  <c:v>131857</c:v>
                 </c:pt>
                 <c:pt idx="129">
-                  <c:v>131441</c:v>
+                  <c:v>131408</c:v>
                 </c:pt>
                 <c:pt idx="130">
-                  <c:v>130995</c:v>
+                  <c:v>130963</c:v>
                 </c:pt>
                 <c:pt idx="131">
-                  <c:v>130553</c:v>
+                  <c:v>130520</c:v>
                 </c:pt>
                 <c:pt idx="132">
-                  <c:v>130113</c:v>
+                  <c:v>130080</c:v>
                 </c:pt>
                 <c:pt idx="133">
-                  <c:v>129676</c:v>
+                  <c:v>129644</c:v>
                 </c:pt>
                 <c:pt idx="134">
-                  <c:v>129243</c:v>
+                  <c:v>129211</c:v>
                 </c:pt>
                 <c:pt idx="135">
-                  <c:v>128813</c:v>
+                  <c:v>128780</c:v>
                 </c:pt>
                 <c:pt idx="136">
-                  <c:v>128386</c:v>
+                  <c:v>128354</c:v>
                 </c:pt>
                 <c:pt idx="137">
-                  <c:v>127962</c:v>
+                  <c:v>127930</c:v>
                 </c:pt>
                 <c:pt idx="138">
-                  <c:v>127542</c:v>
+                  <c:v>127509</c:v>
                 </c:pt>
                 <c:pt idx="139">
-                  <c:v>127125</c:v>
+                  <c:v>127092</c:v>
                 </c:pt>
                 <c:pt idx="140">
-                  <c:v>126711</c:v>
+                  <c:v>126679</c:v>
                 </c:pt>
                 <c:pt idx="141">
-                  <c:v>126301</c:v>
+                  <c:v>126268</c:v>
                 </c:pt>
                 <c:pt idx="142">
-                  <c:v>125894</c:v>
+                  <c:v>125861</c:v>
                 </c:pt>
                 <c:pt idx="143">
-                  <c:v>125490</c:v>
+                  <c:v>125458</c:v>
                 </c:pt>
                 <c:pt idx="144">
-                  <c:v>125090</c:v>
+                  <c:v>125058</c:v>
                 </c:pt>
                 <c:pt idx="145">
-                  <c:v>124693</c:v>
+                  <c:v>124661</c:v>
                 </c:pt>
                 <c:pt idx="146">
-                  <c:v>124300</c:v>
+                  <c:v>124268</c:v>
                 </c:pt>
                 <c:pt idx="147">
-                  <c:v>123910</c:v>
+                  <c:v>123879</c:v>
                 </c:pt>
                 <c:pt idx="148">
-                  <c:v>123524</c:v>
+                  <c:v>123493</c:v>
                 </c:pt>
                 <c:pt idx="149">
-                  <c:v>123142</c:v>
+                  <c:v>123110</c:v>
                 </c:pt>
                 <c:pt idx="150">
-                  <c:v>122763</c:v>
+                  <c:v>122731</c:v>
                 </c:pt>
                 <c:pt idx="151">
-                  <c:v>122387</c:v>
+                  <c:v>122356</c:v>
                 </c:pt>
                 <c:pt idx="152">
-                  <c:v>122016</c:v>
+                  <c:v>121984</c:v>
                 </c:pt>
                 <c:pt idx="153">
-                  <c:v>121647</c:v>
+                  <c:v>121616</c:v>
                 </c:pt>
                 <c:pt idx="154">
-                  <c:v>121283</c:v>
+                  <c:v>121252</c:v>
                 </c:pt>
                 <c:pt idx="155">
-                  <c:v>120922</c:v>
+                  <c:v>120891</c:v>
                 </c:pt>
                 <c:pt idx="156">
-                  <c:v>120565</c:v>
+                  <c:v>120534</c:v>
                 </c:pt>
                 <c:pt idx="157">
-                  <c:v>120212</c:v>
+                  <c:v>120181</c:v>
                 </c:pt>
                 <c:pt idx="158">
-                  <c:v>119862</c:v>
+                  <c:v>119832</c:v>
                 </c:pt>
                 <c:pt idx="159">
-                  <c:v>119516</c:v>
+                  <c:v>119486</c:v>
                 </c:pt>
                 <c:pt idx="160">
-                  <c:v>119174</c:v>
+                  <c:v>119144</c:v>
                 </c:pt>
                 <c:pt idx="161">
-                  <c:v>118835</c:v>
+                  <c:v>118806</c:v>
                 </c:pt>
                 <c:pt idx="162">
-                  <c:v>118501</c:v>
+                  <c:v>118471</c:v>
                 </c:pt>
                 <c:pt idx="163">
-                  <c:v>118170</c:v>
+                  <c:v>118140</c:v>
                 </c:pt>
                 <c:pt idx="164">
-                  <c:v>117843</c:v>
+                  <c:v>117813</c:v>
                 </c:pt>
                 <c:pt idx="165">
-                  <c:v>117519</c:v>
+                  <c:v>117490</c:v>
                 </c:pt>
                 <c:pt idx="166">
-                  <c:v>117200</c:v>
+                  <c:v>117171</c:v>
                 </c:pt>
                 <c:pt idx="167">
-                  <c:v>116884</c:v>
+                  <c:v>116855</c:v>
                 </c:pt>
                 <c:pt idx="168">
-                  <c:v>116572</c:v>
+                  <c:v>116543</c:v>
                 </c:pt>
                 <c:pt idx="169">
-                  <c:v>116263</c:v>
+                  <c:v>116235</c:v>
                 </c:pt>
                 <c:pt idx="170">
-                  <c:v>115959</c:v>
+                  <c:v>115931</c:v>
                 </c:pt>
                 <c:pt idx="171">
-                  <c:v>115658</c:v>
+                  <c:v>115630</c:v>
                 </c:pt>
                 <c:pt idx="172">
-                  <c:v>115361</c:v>
+                  <c:v>115334</c:v>
                 </c:pt>
                 <c:pt idx="173">
-                  <c:v>115068</c:v>
+                  <c:v>115041</c:v>
                 </c:pt>
                 <c:pt idx="174">
-                  <c:v>114779</c:v>
+                  <c:v>114752</c:v>
                 </c:pt>
                 <c:pt idx="175">
-                  <c:v>114493</c:v>
+                  <c:v>114466</c:v>
                 </c:pt>
                 <c:pt idx="176">
-                  <c:v>114212</c:v>
+                  <c:v>114185</c:v>
                 </c:pt>
                 <c:pt idx="177">
-                  <c:v>113934</c:v>
+                  <c:v>113907</c:v>
                 </c:pt>
                 <c:pt idx="178">
-                  <c:v>113659</c:v>
+                  <c:v>113633</c:v>
                 </c:pt>
                 <c:pt idx="179">
-                  <c:v>113389</c:v>
+                  <c:v>113363</c:v>
                 </c:pt>
                 <c:pt idx="180">
-                  <c:v>113122</c:v>
+                  <c:v>113096</c:v>
                 </c:pt>
                 <c:pt idx="181">
-                  <c:v>112859</c:v>
+                  <c:v>112833</c:v>
                 </c:pt>
                 <c:pt idx="182">
-                  <c:v>112600</c:v>
+                  <c:v>112574</c:v>
                 </c:pt>
                 <c:pt idx="183">
-                  <c:v>112344</c:v>
+                  <c:v>112319</c:v>
                 </c:pt>
                 <c:pt idx="184">
-                  <c:v>112092</c:v>
+                  <c:v>112067</c:v>
                 </c:pt>
                 <c:pt idx="185">
-                  <c:v>111844</c:v>
+                  <c:v>111819</c:v>
                 </c:pt>
                 <c:pt idx="186">
-                  <c:v>111599</c:v>
+                  <c:v>111575</c:v>
                 </c:pt>
                 <c:pt idx="187">
-                  <c:v>111358</c:v>
+                  <c:v>111334</c:v>
                 </c:pt>
                 <c:pt idx="188">
-                  <c:v>111121</c:v>
+                  <c:v>111097</c:v>
                 </c:pt>
                 <c:pt idx="189">
-                  <c:v>110887</c:v>
+                  <c:v>110863</c:v>
                 </c:pt>
                 <c:pt idx="190">
-                  <c:v>110657</c:v>
+                  <c:v>110633</c:v>
                 </c:pt>
                 <c:pt idx="191">
-                  <c:v>110430</c:v>
+                  <c:v>110407</c:v>
                 </c:pt>
                 <c:pt idx="192">
-                  <c:v>110207</c:v>
+                  <c:v>110184</c:v>
                 </c:pt>
                 <c:pt idx="193">
-                  <c:v>109987</c:v>
+                  <c:v>109965</c:v>
                 </c:pt>
                 <c:pt idx="194">
-                  <c:v>109771</c:v>
+                  <c:v>109749</c:v>
                 </c:pt>
                 <c:pt idx="195">
-                  <c:v>109559</c:v>
+                  <c:v>109536</c:v>
                 </c:pt>
                 <c:pt idx="196">
-                  <c:v>109350</c:v>
+                  <c:v>109328</c:v>
                 </c:pt>
                 <c:pt idx="197">
-                  <c:v>109144</c:v>
+                  <c:v>109122</c:v>
                 </c:pt>
                 <c:pt idx="198">
-                  <c:v>108941</c:v>
+                  <c:v>108920</c:v>
                 </c:pt>
                 <c:pt idx="199">
-                  <c:v>108743</c:v>
+                  <c:v>108721</c:v>
                 </c:pt>
                 <c:pt idx="200">
-                  <c:v>108547</c:v>
+                  <c:v>108526</c:v>
                 </c:pt>
                 <c:pt idx="201">
-                  <c:v>108355</c:v>
+                  <c:v>108334</c:v>
                 </c:pt>
                 <c:pt idx="202">
-                  <c:v>108166</c:v>
+                  <c:v>108145</c:v>
                 </c:pt>
                 <c:pt idx="203">
-                  <c:v>107980</c:v>
+                  <c:v>107960</c:v>
                 </c:pt>
                 <c:pt idx="204">
-                  <c:v>107797</c:v>
+                  <c:v>107778</c:v>
                 </c:pt>
                 <c:pt idx="205">
-                  <c:v>107618</c:v>
+                  <c:v>107598</c:v>
                 </c:pt>
                 <c:pt idx="206">
-                  <c:v>107442</c:v>
+                  <c:v>107423</c:v>
                 </c:pt>
                 <c:pt idx="207">
-                  <c:v>107269</c:v>
+                  <c:v>107250</c:v>
                 </c:pt>
                 <c:pt idx="208">
-                  <c:v>107099</c:v>
+                  <c:v>107080</c:v>
                 </c:pt>
                 <c:pt idx="209">
-                  <c:v>106932</c:v>
+                  <c:v>106914</c:v>
                 </c:pt>
                 <c:pt idx="210">
-                  <c:v>106768</c:v>
+                  <c:v>106750</c:v>
                 </c:pt>
                 <c:pt idx="211">
-                  <c:v>106607</c:v>
+                  <c:v>106590</c:v>
                 </c:pt>
                 <c:pt idx="212">
-                  <c:v>106450</c:v>
+                  <c:v>106432</c:v>
                 </c:pt>
                 <c:pt idx="213">
-                  <c:v>106295</c:v>
+                  <c:v>106277</c:v>
                 </c:pt>
                 <c:pt idx="214">
-                  <c:v>106143</c:v>
+                  <c:v>106126</c:v>
                 </c:pt>
                 <c:pt idx="215">
-                  <c:v>105994</c:v>
+                  <c:v>105977</c:v>
                 </c:pt>
                 <c:pt idx="216">
-                  <c:v>105847</c:v>
+                  <c:v>105831</c:v>
                 </c:pt>
                 <c:pt idx="217">
-                  <c:v>105704</c:v>
+                  <c:v>105688</c:v>
                 </c:pt>
                 <c:pt idx="218">
-                  <c:v>105563</c:v>
+                  <c:v>105547</c:v>
                 </c:pt>
                 <c:pt idx="219">
-                  <c:v>105425</c:v>
+                  <c:v>105409</c:v>
                 </c:pt>
                 <c:pt idx="220">
-                  <c:v>105290</c:v>
+                  <c:v>105274</c:v>
                 </c:pt>
                 <c:pt idx="221">
-                  <c:v>105157</c:v>
+                  <c:v>105142</c:v>
                 </c:pt>
                 <c:pt idx="222">
-                  <c:v>105027</c:v>
+                  <c:v>105012</c:v>
                 </c:pt>
                 <c:pt idx="223">
-                  <c:v>104900</c:v>
+                  <c:v>104885</c:v>
                 </c:pt>
                 <c:pt idx="224">
-                  <c:v>104775</c:v>
+                  <c:v>104760</c:v>
                 </c:pt>
                 <c:pt idx="225">
-                  <c:v>104652</c:v>
+                  <c:v>104638</c:v>
                 </c:pt>
                 <c:pt idx="226">
-                  <c:v>104533</c:v>
+                  <c:v>104519</c:v>
                 </c:pt>
                 <c:pt idx="227">
-                  <c:v>104415</c:v>
+                  <c:v>104401</c:v>
                 </c:pt>
                 <c:pt idx="228">
-                  <c:v>104300</c:v>
+                  <c:v>104287</c:v>
                 </c:pt>
                 <c:pt idx="229">
-                  <c:v>104187</c:v>
+                  <c:v>104174</c:v>
                 </c:pt>
                 <c:pt idx="230">
-                  <c:v>104077</c:v>
+                  <c:v>104064</c:v>
                 </c:pt>
                 <c:pt idx="231">
-                  <c:v>103969</c:v>
+                  <c:v>103956</c:v>
                 </c:pt>
                 <c:pt idx="232">
-                  <c:v>103863</c:v>
+                  <c:v>103850</c:v>
                 </c:pt>
                 <c:pt idx="233">
-                  <c:v>103759</c:v>
+                  <c:v>103747</c:v>
                 </c:pt>
                 <c:pt idx="234">
-                  <c:v>103658</c:v>
+                  <c:v>103646</c:v>
                 </c:pt>
                 <c:pt idx="235">
-                  <c:v>103558</c:v>
+                  <c:v>103546</c:v>
                 </c:pt>
                 <c:pt idx="236">
-                  <c:v>103461</c:v>
+                  <c:v>103449</c:v>
                 </c:pt>
                 <c:pt idx="237">
-                  <c:v>103366</c:v>
+                  <c:v>103354</c:v>
                 </c:pt>
                 <c:pt idx="238">
-                  <c:v>103272</c:v>
+                  <c:v>103261</c:v>
                 </c:pt>
                 <c:pt idx="239">
-                  <c:v>103181</c:v>
+                  <c:v>103170</c:v>
                 </c:pt>
                 <c:pt idx="240">
-                  <c:v>103092</c:v>
+                  <c:v>103081</c:v>
                 </c:pt>
                 <c:pt idx="241">
-                  <c:v>103004</c:v>
+                  <c:v>102994</c:v>
                 </c:pt>
                 <c:pt idx="242">
-                  <c:v>102919</c:v>
+                  <c:v>102909</c:v>
                 </c:pt>
                 <c:pt idx="243">
-                  <c:v>102835</c:v>
+                  <c:v>102825</c:v>
                 </c:pt>
                 <c:pt idx="244">
-                  <c:v>102753</c:v>
+                  <c:v>102743</c:v>
                 </c:pt>
                 <c:pt idx="245">
-                  <c:v>102673</c:v>
+                  <c:v>102664</c:v>
                 </c:pt>
                 <c:pt idx="246">
-                  <c:v>102595</c:v>
+                  <c:v>102585</c:v>
                 </c:pt>
                 <c:pt idx="247">
-                  <c:v>102518</c:v>
+                  <c:v>102509</c:v>
                 </c:pt>
                 <c:pt idx="248">
-                  <c:v>102443</c:v>
+                  <c:v>102434</c:v>
                 </c:pt>
                 <c:pt idx="249">
-                  <c:v>102369</c:v>
+                  <c:v>102361</c:v>
                 </c:pt>
                 <c:pt idx="250">
-                  <c:v>102297</c:v>
+                  <c:v>102289</c:v>
                 </c:pt>
                 <c:pt idx="251">
-                  <c:v>102227</c:v>
+                  <c:v>102219</c:v>
                 </c:pt>
                 <c:pt idx="252">
-                  <c:v>102158</c:v>
+                  <c:v>102150</c:v>
                 </c:pt>
                 <c:pt idx="253">
-                  <c:v>102091</c:v>
+                  <c:v>102083</c:v>
                 </c:pt>
                 <c:pt idx="254">
-                  <c:v>102025</c:v>
+                  <c:v>102017</c:v>
                 </c:pt>
                 <c:pt idx="255">
-                  <c:v>101960</c:v>
+                  <c:v>101953</c:v>
                 </c:pt>
                 <c:pt idx="256">
-                  <c:v>101897</c:v>
+                  <c:v>101889</c:v>
                 </c:pt>
                 <c:pt idx="257">
-                  <c:v>101835</c:v>
+                  <c:v>101828</c:v>
                 </c:pt>
                 <c:pt idx="258">
-                  <c:v>101774</c:v>
+                  <c:v>101767</c:v>
                 </c:pt>
                 <c:pt idx="259">
-                  <c:v>101715</c:v>
+                  <c:v>101708</c:v>
                 </c:pt>
                 <c:pt idx="260">
-                  <c:v>101657</c:v>
+                  <c:v>101650</c:v>
                 </c:pt>
                 <c:pt idx="261">
-                  <c:v>101600</c:v>
+                  <c:v>101593</c:v>
                 </c:pt>
                 <c:pt idx="262">
-                  <c:v>101544</c:v>
+                  <c:v>101538</c:v>
                 </c:pt>
                 <c:pt idx="263">
-                  <c:v>101489</c:v>
+                  <c:v>101483</c:v>
                 </c:pt>
                 <c:pt idx="264">
-                  <c:v>101436</c:v>
+                  <c:v>101430</c:v>
                 </c:pt>
                 <c:pt idx="265">
-                  <c:v>101383</c:v>
+                  <c:v>101378</c:v>
                 </c:pt>
                 <c:pt idx="266">
-                  <c:v>101332</c:v>
+                  <c:v>101326</c:v>
                 </c:pt>
                 <c:pt idx="267">
-                  <c:v>101281</c:v>
+                  <c:v>101276</c:v>
                 </c:pt>
                 <c:pt idx="268">
-                  <c:v>101231</c:v>
+                  <c:v>101227</c:v>
                 </c:pt>
                 <c:pt idx="269">
-                  <c:v>101183</c:v>
+                  <c:v>101178</c:v>
                 </c:pt>
                 <c:pt idx="270">
-                  <c:v>101135</c:v>
+                  <c:v>101131</c:v>
                 </c:pt>
                 <c:pt idx="271">
-                  <c:v>101088</c:v>
+                  <c:v>101084</c:v>
                 </c:pt>
                 <c:pt idx="272">
-                  <c:v>101042</c:v>
+                  <c:v>101038</c:v>
                 </c:pt>
                 <c:pt idx="273">
-                  <c:v>100997</c:v>
+                  <c:v>100993</c:v>
                 </c:pt>
                 <c:pt idx="274">
-                  <c:v>100952</c:v>
+                  <c:v>100948</c:v>
                 </c:pt>
                 <c:pt idx="275">
-                  <c:v>100909</c:v>
+                  <c:v>100905</c:v>
                 </c:pt>
                 <c:pt idx="276">
-                  <c:v>100866</c:v>
+                  <c:v>100862</c:v>
                 </c:pt>
                 <c:pt idx="277">
-                  <c:v>100823</c:v>
+                  <c:v>100820</c:v>
                 </c:pt>
                 <c:pt idx="278">
-                  <c:v>100781</c:v>
+                  <c:v>100778</c:v>
                 </c:pt>
                 <c:pt idx="279">
-                  <c:v>100740</c:v>
+                  <c:v>100737</c:v>
                 </c:pt>
                 <c:pt idx="280">
-                  <c:v>100700</c:v>
+                  <c:v>100697</c:v>
                 </c:pt>
                 <c:pt idx="281">
-                  <c:v>100660</c:v>
+                  <c:v>100657</c:v>
                 </c:pt>
                 <c:pt idx="282">
-                  <c:v>100620</c:v>
+                  <c:v>100618</c:v>
                 </c:pt>
                 <c:pt idx="283">
-                  <c:v>100581</c:v>
+                  <c:v>100579</c:v>
                 </c:pt>
                 <c:pt idx="284">
-                  <c:v>100543</c:v>
+                  <c:v>100541</c:v>
                 </c:pt>
                 <c:pt idx="285">
-                  <c:v>100505</c:v>
+                  <c:v>100503</c:v>
                 </c:pt>
                 <c:pt idx="286">
-                  <c:v>100467</c:v>
+                  <c:v>100465</c:v>
                 </c:pt>
                 <c:pt idx="287">
-                  <c:v>100430</c:v>
+                  <c:v>100428</c:v>
                 </c:pt>
                 <c:pt idx="288">
-                  <c:v>100393</c:v>
+                  <c:v>100391</c:v>
                 </c:pt>
                 <c:pt idx="289">
-                  <c:v>100356</c:v>
+                  <c:v>100355</c:v>
                 </c:pt>
                 <c:pt idx="290">
-                  <c:v>100320</c:v>
+                  <c:v>100318</c:v>
                 </c:pt>
                 <c:pt idx="291">
-                  <c:v>100284</c:v>
+                  <c:v>100282</c:v>
                 </c:pt>
                 <c:pt idx="292">
-                  <c:v>100248</c:v>
+                  <c:v>100247</c:v>
                 </c:pt>
                 <c:pt idx="293">
-                  <c:v>100212</c:v>
+                  <c:v>100211</c:v>
                 </c:pt>
                 <c:pt idx="294">
                   <c:v>100176</c:v>
                 </c:pt>
                 <c:pt idx="295">
-                  <c:v>100141</c:v>
+                  <c:v>100140</c:v>
                 </c:pt>
                 <c:pt idx="296">
-                  <c:v>100106</c:v>
+                  <c:v>100105</c:v>
                 </c:pt>
                 <c:pt idx="297">
                   <c:v>100070</c:v>
@@ -2793,7 +2793,7 @@
         <v>3.3444799999999999E-4</v>
       </c>
       <c r="F5">
-        <v>199494</v>
+        <v>199489</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.3">
@@ -2807,7 +2807,7 @@
         <v>6.6889599999999999E-4</v>
       </c>
       <c r="F6">
-        <v>198977</v>
+        <v>198971</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
@@ -2821,7 +2821,7 @@
         <v>1.0033399999999999E-3</v>
       </c>
       <c r="F7">
-        <v>198456</v>
+        <v>198449</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.3">
@@ -2835,7 +2835,7 @@
         <v>1.3377899999999999E-3</v>
       </c>
       <c r="F8">
-        <v>197933</v>
+        <v>197926</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.3">
@@ -2849,7 +2849,7 @@
         <v>1.67224E-3</v>
       </c>
       <c r="F9">
-        <v>197409</v>
+        <v>197402</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.3">
@@ -2863,7 +2863,7 @@
         <v>2.0066900000000002E-3</v>
       </c>
       <c r="F10">
-        <v>196884</v>
+        <v>196877</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.3">
@@ -2877,7 +2877,7 @@
         <v>2.3411399999999998E-3</v>
       </c>
       <c r="F11">
-        <v>196357</v>
+        <v>196350</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.3">
@@ -2891,7 +2891,7 @@
         <v>2.6755899999999998E-3</v>
       </c>
       <c r="F12">
-        <v>195830</v>
+        <v>195822</v>
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.3">
@@ -2905,7 +2905,7 @@
         <v>3.0100299999999999E-3</v>
       </c>
       <c r="F13">
-        <v>195301</v>
+        <v>195293</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.3">
@@ -2919,7 +2919,7 @@
         <v>3.3444799999999999E-3</v>
       </c>
       <c r="F14">
-        <v>194771</v>
+        <v>194763</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.3">
@@ -2933,7 +2933,7 @@
         <v>3.67893E-3</v>
       </c>
       <c r="F15">
-        <v>194239</v>
+        <v>194231</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.3">
@@ -2947,7 +2947,7 @@
         <v>4.0133800000000004E-3</v>
       </c>
       <c r="F16">
-        <v>193707</v>
+        <v>193698</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.3">
@@ -2961,7 +2961,7 @@
         <v>4.3478299999999996E-3</v>
       </c>
       <c r="F17">
-        <v>193174</v>
+        <v>193165</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.3">
@@ -2975,7 +2975,7 @@
         <v>4.6822699999999997E-3</v>
       </c>
       <c r="F18">
-        <v>192639</v>
+        <v>192630</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.3">
@@ -2989,7 +2989,7 @@
         <v>5.0167199999999997E-3</v>
       </c>
       <c r="F19">
-        <v>192103</v>
+        <v>192094</v>
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.3">
@@ -3003,7 +3003,7 @@
         <v>5.3511699999999997E-3</v>
       </c>
       <c r="F20">
-        <v>191566</v>
+        <v>191557</v>
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.3">
@@ -3017,7 +3017,7 @@
         <v>5.6856199999999997E-3</v>
       </c>
       <c r="F21">
-        <v>191029</v>
+        <v>191019</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.3">
@@ -3031,7 +3031,7 @@
         <v>6.0200699999999998E-3</v>
       </c>
       <c r="F22">
-        <v>190490</v>
+        <v>190480</v>
       </c>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.3">
@@ -3045,7 +3045,7 @@
         <v>6.3545199999999998E-3</v>
       </c>
       <c r="F23">
-        <v>189950</v>
+        <v>189940</v>
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.3">
@@ -3059,7 +3059,7 @@
         <v>6.6889599999999999E-3</v>
       </c>
       <c r="F24">
-        <v>189409</v>
+        <v>189398</v>
       </c>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.3">
@@ -3073,7 +3073,7 @@
         <v>7.0234099999999999E-3</v>
       </c>
       <c r="F25">
-        <v>188867</v>
+        <v>188856</v>
       </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.3">
@@ -3087,7 +3087,7 @@
         <v>7.3578599999999999E-3</v>
       </c>
       <c r="F26">
-        <v>188325</v>
+        <v>188314</v>
       </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.3">
@@ -3101,7 +3101,7 @@
         <v>7.6923099999999999E-3</v>
       </c>
       <c r="F27">
-        <v>187781</v>
+        <v>187770</v>
       </c>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.3">
@@ -3115,7 +3115,7 @@
         <v>8.0267600000000008E-3</v>
       </c>
       <c r="F28">
-        <v>187237</v>
+        <v>187225</v>
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.3">
@@ -3129,7 +3129,7 @@
         <v>8.3611999999999992E-3</v>
       </c>
       <c r="F29">
-        <v>186691</v>
+        <v>186679</v>
       </c>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.3">
@@ -3143,7 +3143,7 @@
         <v>8.6956499999999992E-3</v>
       </c>
       <c r="F30">
-        <v>186145</v>
+        <v>186133</v>
       </c>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.3">
@@ -3157,7 +3157,7 @@
         <v>9.0300999999999992E-3</v>
       </c>
       <c r="F31">
-        <v>185598</v>
+        <v>185586</v>
       </c>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.3">
@@ -3171,7 +3171,7 @@
         <v>9.3645499999999993E-3</v>
       </c>
       <c r="F32">
-        <v>185050</v>
+        <v>185037</v>
       </c>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.3">
@@ -3185,7 +3185,7 @@
         <v>9.6989999999999993E-3</v>
       </c>
       <c r="F33">
-        <v>184502</v>
+        <v>184489</v>
       </c>
     </row>
     <row r="34" spans="2:6" x14ac:dyDescent="0.3">
@@ -3199,7 +3199,7 @@
         <v>1.00334E-2</v>
       </c>
       <c r="F34">
-        <v>183952</v>
+        <v>183939</v>
       </c>
     </row>
     <row r="35" spans="2:6" x14ac:dyDescent="0.3">
@@ -3213,7 +3213,7 @@
         <v>1.0367899999999999E-2</v>
       </c>
       <c r="F35">
-        <v>183402</v>
+        <v>183389</v>
       </c>
     </row>
     <row r="36" spans="2:6" x14ac:dyDescent="0.3">
@@ -3227,7 +3227,7 @@
         <v>1.07023E-2</v>
       </c>
       <c r="F36">
-        <v>182851</v>
+        <v>182838</v>
       </c>
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.3">
@@ -3241,7 +3241,7 @@
         <v>1.1036799999999999E-2</v>
       </c>
       <c r="F37">
-        <v>182300</v>
+        <v>182286</v>
       </c>
     </row>
     <row r="38" spans="2:6" x14ac:dyDescent="0.3">
@@ -3255,7 +3255,7 @@
         <v>1.13712E-2</v>
       </c>
       <c r="F38">
-        <v>181748</v>
+        <v>181734</v>
       </c>
     </row>
     <row r="39" spans="2:6" x14ac:dyDescent="0.3">
@@ -3269,7 +3269,7 @@
         <v>1.1705699999999999E-2</v>
       </c>
       <c r="F39">
-        <v>181195</v>
+        <v>181181</v>
       </c>
     </row>
     <row r="40" spans="2:6" x14ac:dyDescent="0.3">
@@ -3283,7 +3283,7 @@
         <v>1.20401E-2</v>
       </c>
       <c r="F40">
-        <v>180642</v>
+        <v>180627</v>
       </c>
     </row>
     <row r="41" spans="2:6" x14ac:dyDescent="0.3">
@@ -3297,7 +3297,7 @@
         <v>1.2374599999999999E-2</v>
       </c>
       <c r="F41">
-        <v>180088</v>
+        <v>180073</v>
       </c>
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.3">
@@ -3311,7 +3311,7 @@
         <v>1.2709E-2</v>
       </c>
       <c r="F42">
-        <v>179534</v>
+        <v>179519</v>
       </c>
     </row>
     <row r="43" spans="2:6" x14ac:dyDescent="0.3">
@@ -3325,7 +3325,7 @@
         <v>1.30435E-2</v>
       </c>
       <c r="F43">
-        <v>178979</v>
+        <v>178964</v>
       </c>
     </row>
     <row r="44" spans="2:6" x14ac:dyDescent="0.3">
@@ -3333,7 +3333,7 @@
         <v>1.33779E-2</v>
       </c>
       <c r="F44">
-        <v>178424</v>
+        <v>178408</v>
       </c>
     </row>
     <row r="45" spans="2:6" x14ac:dyDescent="0.3">
@@ -3341,7 +3341,7 @@
         <v>1.37124E-2</v>
       </c>
       <c r="F45">
-        <v>177868</v>
+        <v>177852</v>
       </c>
     </row>
     <row r="46" spans="2:6" x14ac:dyDescent="0.3">
@@ -3349,7 +3349,7 @@
         <v>1.40468E-2</v>
       </c>
       <c r="F46">
-        <v>177312</v>
+        <v>177296</v>
       </c>
     </row>
     <row r="47" spans="2:6" x14ac:dyDescent="0.3">
@@ -3357,7 +3357,7 @@
         <v>1.43813E-2</v>
       </c>
       <c r="F47">
-        <v>176756</v>
+        <v>176739</v>
       </c>
     </row>
     <row r="48" spans="2:6" x14ac:dyDescent="0.3">
@@ -3365,7 +3365,7 @@
         <v>1.47157E-2</v>
       </c>
       <c r="F48">
-        <v>176199</v>
+        <v>176182</v>
       </c>
     </row>
     <row r="49" spans="5:6" x14ac:dyDescent="0.3">
@@ -3373,7 +3373,7 @@
         <v>1.50502E-2</v>
       </c>
       <c r="F49">
-        <v>175642</v>
+        <v>175625</v>
       </c>
     </row>
     <row r="50" spans="5:6" x14ac:dyDescent="0.3">
@@ -3381,7 +3381,7 @@
         <v>1.53846E-2</v>
       </c>
       <c r="F50">
-        <v>175084</v>
+        <v>175067</v>
       </c>
     </row>
     <row r="51" spans="5:6" x14ac:dyDescent="0.3">
@@ -3389,7 +3389,7 @@
         <v>1.57191E-2</v>
       </c>
       <c r="F51">
-        <v>174527</v>
+        <v>174509</v>
       </c>
     </row>
     <row r="52" spans="5:6" x14ac:dyDescent="0.3">
@@ -3397,7 +3397,7 @@
         <v>1.6053499999999998E-2</v>
       </c>
       <c r="F52">
-        <v>173969</v>
+        <v>173951</v>
       </c>
     </row>
     <row r="53" spans="5:6" x14ac:dyDescent="0.3">
@@ -3405,7 +3405,7 @@
         <v>1.6388E-2</v>
       </c>
       <c r="F53">
-        <v>173410</v>
+        <v>173392</v>
       </c>
     </row>
     <row r="54" spans="5:6" x14ac:dyDescent="0.3">
@@ -3413,7 +3413,7 @@
         <v>1.6722399999999998E-2</v>
       </c>
       <c r="F54">
-        <v>172852</v>
+        <v>172834</v>
       </c>
     </row>
     <row r="55" spans="5:6" x14ac:dyDescent="0.3">
@@ -3421,7 +3421,7 @@
         <v>1.70569E-2</v>
       </c>
       <c r="F55">
-        <v>172294</v>
+        <v>172275</v>
       </c>
     </row>
     <row r="56" spans="5:6" x14ac:dyDescent="0.3">
@@ -3429,7 +3429,7 @@
         <v>1.7391299999999998E-2</v>
       </c>
       <c r="F56">
-        <v>171735</v>
+        <v>171716</v>
       </c>
     </row>
     <row r="57" spans="5:6" x14ac:dyDescent="0.3">
@@ -3437,7 +3437,7 @@
         <v>1.77258E-2</v>
       </c>
       <c r="F57">
-        <v>171176</v>
+        <v>171157</v>
       </c>
     </row>
     <row r="58" spans="5:6" x14ac:dyDescent="0.3">
@@ -3445,7 +3445,7 @@
         <v>1.8060199999999998E-2</v>
       </c>
       <c r="F58">
-        <v>170618</v>
+        <v>170598</v>
       </c>
     </row>
     <row r="59" spans="5:6" x14ac:dyDescent="0.3">
@@ -3453,7 +3453,7 @@
         <v>1.8394600000000001E-2</v>
       </c>
       <c r="F59">
-        <v>170059</v>
+        <v>170039</v>
       </c>
     </row>
     <row r="60" spans="5:6" x14ac:dyDescent="0.3">
@@ -3461,7 +3461,7 @@
         <v>1.8729099999999999E-2</v>
       </c>
       <c r="F60">
-        <v>169501</v>
+        <v>169480</v>
       </c>
     </row>
     <row r="61" spans="5:6" x14ac:dyDescent="0.3">
@@ -3469,7 +3469,7 @@
         <v>1.9063500000000001E-2</v>
       </c>
       <c r="F61">
-        <v>168942</v>
+        <v>168921</v>
       </c>
     </row>
     <row r="62" spans="5:6" x14ac:dyDescent="0.3">
@@ -3477,7 +3477,7 @@
         <v>1.9397999999999999E-2</v>
       </c>
       <c r="F62">
-        <v>168384</v>
+        <v>168363</v>
       </c>
     </row>
     <row r="63" spans="5:6" x14ac:dyDescent="0.3">
@@ -3485,7 +3485,7 @@
         <v>1.9732400000000001E-2</v>
       </c>
       <c r="F63">
-        <v>167825</v>
+        <v>167804</v>
       </c>
     </row>
     <row r="64" spans="5:6" x14ac:dyDescent="0.3">
@@ -3493,7 +3493,7 @@
         <v>2.0066899999999999E-2</v>
       </c>
       <c r="F64">
-        <v>167267</v>
+        <v>167246</v>
       </c>
     </row>
     <row r="65" spans="5:6" x14ac:dyDescent="0.3">
@@ -3501,7 +3501,7 @@
         <v>2.0401300000000001E-2</v>
       </c>
       <c r="F65">
-        <v>166709</v>
+        <v>166688</v>
       </c>
     </row>
     <row r="66" spans="5:6" x14ac:dyDescent="0.3">
@@ -3509,7 +3509,7 @@
         <v>2.0735799999999999E-2</v>
       </c>
       <c r="F66">
-        <v>166151</v>
+        <v>166130</v>
       </c>
     </row>
     <row r="67" spans="5:6" x14ac:dyDescent="0.3">
@@ -3517,7 +3517,7 @@
         <v>2.1070200000000001E-2</v>
       </c>
       <c r="F67">
-        <v>165594</v>
+        <v>165572</v>
       </c>
     </row>
     <row r="68" spans="5:6" x14ac:dyDescent="0.3">
@@ -3525,7 +3525,7 @@
         <v>2.1404699999999999E-2</v>
       </c>
       <c r="F68">
-        <v>165037</v>
+        <v>165015</v>
       </c>
     </row>
     <row r="69" spans="5:6" x14ac:dyDescent="0.3">
@@ -3533,7 +3533,7 @@
         <v>2.1739100000000001E-2</v>
       </c>
       <c r="F69">
-        <v>164480</v>
+        <v>164458</v>
       </c>
     </row>
     <row r="70" spans="5:6" x14ac:dyDescent="0.3">
@@ -3541,7 +3541,7 @@
         <v>2.2073599999999999E-2</v>
       </c>
       <c r="F70">
-        <v>163924</v>
+        <v>163901</v>
       </c>
     </row>
     <row r="71" spans="5:6" x14ac:dyDescent="0.3">
@@ -3549,7 +3549,7 @@
         <v>2.2408000000000001E-2</v>
       </c>
       <c r="F71">
-        <v>163368</v>
+        <v>163345</v>
       </c>
     </row>
     <row r="72" spans="5:6" x14ac:dyDescent="0.3">
@@ -3557,7 +3557,7 @@
         <v>2.2742499999999999E-2</v>
       </c>
       <c r="F72">
-        <v>162812</v>
+        <v>162789</v>
       </c>
     </row>
     <row r="73" spans="5:6" x14ac:dyDescent="0.3">
@@ -3565,7 +3565,7 @@
         <v>2.3076900000000001E-2</v>
       </c>
       <c r="F73">
-        <v>162257</v>
+        <v>162234</v>
       </c>
     </row>
     <row r="74" spans="5:6" x14ac:dyDescent="0.3">
@@ -3573,7 +3573,7 @@
         <v>2.3411399999999999E-2</v>
       </c>
       <c r="F74">
-        <v>161703</v>
+        <v>161679</v>
       </c>
     </row>
     <row r="75" spans="5:6" x14ac:dyDescent="0.3">
@@ -3581,7 +3581,7 @@
         <v>2.3745800000000001E-2</v>
       </c>
       <c r="F75">
-        <v>161149</v>
+        <v>161125</v>
       </c>
     </row>
     <row r="76" spans="5:6" x14ac:dyDescent="0.3">
@@ -3589,7 +3589,7 @@
         <v>2.4080299999999999E-2</v>
       </c>
       <c r="F76">
-        <v>160596</v>
+        <v>160572</v>
       </c>
     </row>
     <row r="77" spans="5:6" x14ac:dyDescent="0.3">
@@ -3597,7 +3597,7 @@
         <v>2.4414700000000001E-2</v>
       </c>
       <c r="F77">
-        <v>160043</v>
+        <v>160019</v>
       </c>
     </row>
     <row r="78" spans="5:6" x14ac:dyDescent="0.3">
@@ -3605,7 +3605,7 @@
         <v>2.4749199999999999E-2</v>
       </c>
       <c r="F78">
-        <v>159492</v>
+        <v>159467</v>
       </c>
     </row>
     <row r="79" spans="5:6" x14ac:dyDescent="0.3">
@@ -3613,7 +3613,7 @@
         <v>2.5083600000000001E-2</v>
       </c>
       <c r="F79">
-        <v>158940</v>
+        <v>158915</v>
       </c>
     </row>
     <row r="80" spans="5:6" x14ac:dyDescent="0.3">
@@ -3621,7 +3621,7 @@
         <v>2.5418099999999999E-2</v>
       </c>
       <c r="F80">
-        <v>158390</v>
+        <v>158365</v>
       </c>
     </row>
     <row r="81" spans="5:6" x14ac:dyDescent="0.3">
@@ -3629,7 +3629,7 @@
         <v>2.5752500000000001E-2</v>
       </c>
       <c r="F81">
-        <v>157841</v>
+        <v>157815</v>
       </c>
     </row>
     <row r="82" spans="5:6" x14ac:dyDescent="0.3">
@@ -3637,7 +3637,7 @@
         <v>2.6086999999999999E-2</v>
       </c>
       <c r="F82">
-        <v>157292</v>
+        <v>157266</v>
       </c>
     </row>
     <row r="83" spans="5:6" x14ac:dyDescent="0.3">
@@ -3645,7 +3645,7 @@
         <v>2.6421400000000001E-2</v>
       </c>
       <c r="F83">
-        <v>156744</v>
+        <v>156718</v>
       </c>
     </row>
     <row r="84" spans="5:6" x14ac:dyDescent="0.3">
@@ -3653,7 +3653,7 @@
         <v>2.6755899999999999E-2</v>
       </c>
       <c r="F84">
-        <v>156197</v>
+        <v>156171</v>
       </c>
     </row>
     <row r="85" spans="5:6" x14ac:dyDescent="0.3">
@@ -3661,7 +3661,7 @@
         <v>2.7090300000000001E-2</v>
       </c>
       <c r="F85">
-        <v>155652</v>
+        <v>155625</v>
       </c>
     </row>
     <row r="86" spans="5:6" x14ac:dyDescent="0.3">
@@ -3669,7 +3669,7 @@
         <v>2.74247E-2</v>
       </c>
       <c r="F86">
-        <v>155107</v>
+        <v>155080</v>
       </c>
     </row>
     <row r="87" spans="5:6" x14ac:dyDescent="0.3">
@@ -3677,7 +3677,7 @@
         <v>2.7759200000000001E-2</v>
       </c>
       <c r="F87">
-        <v>154563</v>
+        <v>154536</v>
       </c>
     </row>
     <row r="88" spans="5:6" x14ac:dyDescent="0.3">
@@ -3685,7 +3685,7 @@
         <v>2.80936E-2</v>
       </c>
       <c r="F88">
-        <v>154020</v>
+        <v>153993</v>
       </c>
     </row>
     <row r="89" spans="5:6" x14ac:dyDescent="0.3">
@@ -3693,7 +3693,7 @@
         <v>2.8428100000000001E-2</v>
       </c>
       <c r="F89">
-        <v>153479</v>
+        <v>153452</v>
       </c>
     </row>
     <row r="90" spans="5:6" x14ac:dyDescent="0.3">
@@ -3701,7 +3701,7 @@
         <v>2.87625E-2</v>
       </c>
       <c r="F90">
-        <v>152939</v>
+        <v>152911</v>
       </c>
     </row>
     <row r="91" spans="5:6" x14ac:dyDescent="0.3">
@@ -3709,7 +3709,7 @@
         <v>2.9097000000000001E-2</v>
       </c>
       <c r="F91">
-        <v>152400</v>
+        <v>152372</v>
       </c>
     </row>
     <row r="92" spans="5:6" x14ac:dyDescent="0.3">
@@ -3717,7 +3717,7 @@
         <v>2.94314E-2</v>
       </c>
       <c r="F92">
-        <v>151862</v>
+        <v>151834</v>
       </c>
     </row>
     <row r="93" spans="5:6" x14ac:dyDescent="0.3">
@@ -3725,7 +3725,7 @@
         <v>2.9765900000000001E-2</v>
       </c>
       <c r="F93">
-        <v>151325</v>
+        <v>151297</v>
       </c>
     </row>
     <row r="94" spans="5:6" x14ac:dyDescent="0.3">
@@ -3733,7 +3733,7 @@
         <v>3.01003E-2</v>
       </c>
       <c r="F94">
-        <v>150790</v>
+        <v>150762</v>
       </c>
     </row>
     <row r="95" spans="5:6" x14ac:dyDescent="0.3">
@@ -3741,7 +3741,7 @@
         <v>3.0434800000000001E-2</v>
       </c>
       <c r="F95">
-        <v>150257</v>
+        <v>150228</v>
       </c>
     </row>
     <row r="96" spans="5:6" x14ac:dyDescent="0.3">
@@ -3749,7 +3749,7 @@
         <v>3.07692E-2</v>
       </c>
       <c r="F96">
-        <v>149724</v>
+        <v>149696</v>
       </c>
     </row>
     <row r="97" spans="5:6" x14ac:dyDescent="0.3">
@@ -3757,7 +3757,7 @@
         <v>3.1103700000000001E-2</v>
       </c>
       <c r="F97">
-        <v>149194</v>
+        <v>149165</v>
       </c>
     </row>
     <row r="98" spans="5:6" x14ac:dyDescent="0.3">
@@ -3765,7 +3765,7 @@
         <v>3.1438099999999997E-2</v>
       </c>
       <c r="F98">
-        <v>148664</v>
+        <v>148635</v>
       </c>
     </row>
     <row r="99" spans="5:6" x14ac:dyDescent="0.3">
@@ -3773,7 +3773,7 @@
         <v>3.1772599999999998E-2</v>
       </c>
       <c r="F99">
-        <v>148137</v>
+        <v>148107</v>
       </c>
     </row>
     <row r="100" spans="5:6" x14ac:dyDescent="0.3">
@@ -3781,7 +3781,7 @@
         <v>3.2106999999999997E-2</v>
       </c>
       <c r="F100">
-        <v>147611</v>
+        <v>147581</v>
       </c>
     </row>
     <row r="101" spans="5:6" x14ac:dyDescent="0.3">
@@ -3789,7 +3789,7 @@
         <v>3.2441499999999998E-2</v>
       </c>
       <c r="F101">
-        <v>147086</v>
+        <v>147057</v>
       </c>
     </row>
     <row r="102" spans="5:6" x14ac:dyDescent="0.3">
@@ -3797,7 +3797,7 @@
         <v>3.2775899999999997E-2</v>
       </c>
       <c r="F102">
-        <v>146564</v>
+        <v>146534</v>
       </c>
     </row>
     <row r="103" spans="5:6" x14ac:dyDescent="0.3">
@@ -3805,7 +3805,7 @@
         <v>3.3110399999999998E-2</v>
       </c>
       <c r="F103">
-        <v>146043</v>
+        <v>146013</v>
       </c>
     </row>
     <row r="104" spans="5:6" x14ac:dyDescent="0.3">
@@ -3813,7 +3813,7 @@
         <v>3.3444799999999997E-2</v>
       </c>
       <c r="F104">
-        <v>145524</v>
+        <v>145493</v>
       </c>
     </row>
     <row r="105" spans="5:6" x14ac:dyDescent="0.3">
@@ -3821,7 +3821,7 @@
         <v>3.3779299999999998E-2</v>
       </c>
       <c r="F105">
-        <v>145006</v>
+        <v>144976</v>
       </c>
     </row>
     <row r="106" spans="5:6" x14ac:dyDescent="0.3">
@@ -3829,7 +3829,7 @@
         <v>3.4113699999999997E-2</v>
       </c>
       <c r="F106">
-        <v>144491</v>
+        <v>144461</v>
       </c>
     </row>
     <row r="107" spans="5:6" x14ac:dyDescent="0.3">
@@ -3837,7 +3837,7 @@
         <v>3.4448199999999998E-2</v>
       </c>
       <c r="F107">
-        <v>143977</v>
+        <v>143947</v>
       </c>
     </row>
     <row r="108" spans="5:6" x14ac:dyDescent="0.3">
@@ -3845,7 +3845,7 @@
         <v>3.4782599999999997E-2</v>
       </c>
       <c r="F108">
-        <v>143466</v>
+        <v>143435</v>
       </c>
     </row>
     <row r="109" spans="5:6" x14ac:dyDescent="0.3">
@@ -3853,7 +3853,7 @@
         <v>3.5117099999999998E-2</v>
       </c>
       <c r="F109">
-        <v>142956</v>
+        <v>142926</v>
       </c>
     </row>
     <row r="110" spans="5:6" x14ac:dyDescent="0.3">
@@ -3861,7 +3861,7 @@
         <v>3.5451499999999997E-2</v>
       </c>
       <c r="F110">
-        <v>142449</v>
+        <v>142418</v>
       </c>
     </row>
     <row r="111" spans="5:6" x14ac:dyDescent="0.3">
@@ -3869,7 +3869,7 @@
         <v>3.5785999999999998E-2</v>
       </c>
       <c r="F111">
-        <v>141944</v>
+        <v>141913</v>
       </c>
     </row>
     <row r="112" spans="5:6" x14ac:dyDescent="0.3">
@@ -3877,7 +3877,7 @@
         <v>3.6120399999999997E-2</v>
       </c>
       <c r="F112">
-        <v>141440</v>
+        <v>141409</v>
       </c>
     </row>
     <row r="113" spans="5:6" x14ac:dyDescent="0.3">
@@ -3885,7 +3885,7 @@
         <v>3.6454800000000002E-2</v>
       </c>
       <c r="F113">
-        <v>140939</v>
+        <v>140908</v>
       </c>
     </row>
     <row r="114" spans="5:6" x14ac:dyDescent="0.3">
@@ -3893,7 +3893,7 @@
         <v>3.6789299999999997E-2</v>
       </c>
       <c r="F114">
-        <v>140441</v>
+        <v>140409</v>
       </c>
     </row>
     <row r="115" spans="5:6" x14ac:dyDescent="0.3">
@@ -3901,7 +3901,7 @@
         <v>3.7123700000000003E-2</v>
       </c>
       <c r="F115">
-        <v>139944</v>
+        <v>139913</v>
       </c>
     </row>
     <row r="116" spans="5:6" x14ac:dyDescent="0.3">
@@ -3909,7 +3909,7 @@
         <v>3.7458199999999997E-2</v>
       </c>
       <c r="F116">
-        <v>139450</v>
+        <v>139418</v>
       </c>
     </row>
     <row r="117" spans="5:6" x14ac:dyDescent="0.3">
@@ -3917,7 +3917,7 @@
         <v>3.7792600000000003E-2</v>
       </c>
       <c r="F117">
-        <v>138958</v>
+        <v>138926</v>
       </c>
     </row>
     <row r="118" spans="5:6" x14ac:dyDescent="0.3">
@@ -3925,7 +3925,7 @@
         <v>3.8127099999999997E-2</v>
       </c>
       <c r="F118">
-        <v>138468</v>
+        <v>138437</v>
       </c>
     </row>
     <row r="119" spans="5:6" x14ac:dyDescent="0.3">
@@ -3933,7 +3933,7 @@
         <v>3.8461500000000003E-2</v>
       </c>
       <c r="F119">
-        <v>137981</v>
+        <v>137950</v>
       </c>
     </row>
     <row r="120" spans="5:6" x14ac:dyDescent="0.3">
@@ -3941,7 +3941,7 @@
         <v>3.8795999999999997E-2</v>
       </c>
       <c r="F120">
-        <v>137497</v>
+        <v>137465</v>
       </c>
     </row>
     <row r="121" spans="5:6" x14ac:dyDescent="0.3">
@@ -3949,7 +3949,7 @@
         <v>3.9130400000000003E-2</v>
       </c>
       <c r="F121">
-        <v>137015</v>
+        <v>136983</v>
       </c>
     </row>
     <row r="122" spans="5:6" x14ac:dyDescent="0.3">
@@ -3957,7 +3957,7 @@
         <v>3.9464899999999997E-2</v>
       </c>
       <c r="F122">
-        <v>136535</v>
+        <v>136503</v>
       </c>
     </row>
     <row r="123" spans="5:6" x14ac:dyDescent="0.3">
@@ -3965,7 +3965,7 @@
         <v>3.9799300000000003E-2</v>
       </c>
       <c r="F123">
-        <v>136058</v>
+        <v>136026</v>
       </c>
     </row>
     <row r="124" spans="5:6" x14ac:dyDescent="0.3">
@@ -3973,7 +3973,7 @@
         <v>4.0133799999999997E-2</v>
       </c>
       <c r="F124">
-        <v>135584</v>
+        <v>135552</v>
       </c>
     </row>
     <row r="125" spans="5:6" x14ac:dyDescent="0.3">
@@ -3981,7 +3981,7 @@
         <v>4.0468200000000003E-2</v>
       </c>
       <c r="F125">
-        <v>135113</v>
+        <v>135080</v>
       </c>
     </row>
     <row r="126" spans="5:6" x14ac:dyDescent="0.3">
@@ -3989,7 +3989,7 @@
         <v>4.0802699999999997E-2</v>
       </c>
       <c r="F126">
-        <v>134644</v>
+        <v>134611</v>
       </c>
     </row>
     <row r="127" spans="5:6" x14ac:dyDescent="0.3">
@@ -3997,7 +3997,7 @@
         <v>4.1137100000000003E-2</v>
       </c>
       <c r="F127">
-        <v>134178</v>
+        <v>134145</v>
       </c>
     </row>
     <row r="128" spans="5:6" x14ac:dyDescent="0.3">
@@ -4005,7 +4005,7 @@
         <v>4.1471599999999997E-2</v>
       </c>
       <c r="F128">
-        <v>133714</v>
+        <v>133682</v>
       </c>
     </row>
     <row r="129" spans="5:6" x14ac:dyDescent="0.3">
@@ -4013,7 +4013,7 @@
         <v>4.1806000000000003E-2</v>
       </c>
       <c r="F129">
-        <v>133254</v>
+        <v>133221</v>
       </c>
     </row>
     <row r="130" spans="5:6" x14ac:dyDescent="0.3">
@@ -4021,7 +4021,7 @@
         <v>4.2140499999999997E-2</v>
       </c>
       <c r="F130">
-        <v>132796</v>
+        <v>132764</v>
       </c>
     </row>
     <row r="131" spans="5:6" x14ac:dyDescent="0.3">
@@ -4029,7 +4029,7 @@
         <v>4.2474900000000003E-2</v>
       </c>
       <c r="F131">
-        <v>132342</v>
+        <v>132309</v>
       </c>
     </row>
     <row r="132" spans="5:6" x14ac:dyDescent="0.3">
@@ -4037,7 +4037,7 @@
         <v>4.2809399999999997E-2</v>
       </c>
       <c r="F132">
-        <v>131890</v>
+        <v>131857</v>
       </c>
     </row>
     <row r="133" spans="5:6" x14ac:dyDescent="0.3">
@@ -4045,7 +4045,7 @@
         <v>4.3143800000000003E-2</v>
       </c>
       <c r="F133">
-        <v>131441</v>
+        <v>131408</v>
       </c>
     </row>
     <row r="134" spans="5:6" x14ac:dyDescent="0.3">
@@ -4053,7 +4053,7 @@
         <v>4.3478299999999998E-2</v>
       </c>
       <c r="F134">
-        <v>130995</v>
+        <v>130963</v>
       </c>
     </row>
     <row r="135" spans="5:6" x14ac:dyDescent="0.3">
@@ -4061,7 +4061,7 @@
         <v>4.3812700000000003E-2</v>
       </c>
       <c r="F135">
-        <v>130553</v>
+        <v>130520</v>
       </c>
     </row>
     <row r="136" spans="5:6" x14ac:dyDescent="0.3">
@@ -4069,7 +4069,7 @@
         <v>4.4147199999999998E-2</v>
       </c>
       <c r="F136">
-        <v>130113</v>
+        <v>130080</v>
       </c>
     </row>
     <row r="137" spans="5:6" x14ac:dyDescent="0.3">
@@ -4077,7 +4077,7 @@
         <v>4.4481600000000003E-2</v>
       </c>
       <c r="F137">
-        <v>129676</v>
+        <v>129644</v>
       </c>
     </row>
     <row r="138" spans="5:6" x14ac:dyDescent="0.3">
@@ -4085,7 +4085,7 @@
         <v>4.4816099999999998E-2</v>
       </c>
       <c r="F138">
-        <v>129243</v>
+        <v>129211</v>
       </c>
     </row>
     <row r="139" spans="5:6" x14ac:dyDescent="0.3">
@@ -4093,7 +4093,7 @@
         <v>4.5150500000000003E-2</v>
       </c>
       <c r="F139">
-        <v>128813</v>
+        <v>128780</v>
       </c>
     </row>
     <row r="140" spans="5:6" x14ac:dyDescent="0.3">
@@ -4101,7 +4101,7 @@
         <v>4.5484900000000002E-2</v>
       </c>
       <c r="F140">
-        <v>128386</v>
+        <v>128354</v>
       </c>
     </row>
     <row r="141" spans="5:6" x14ac:dyDescent="0.3">
@@ -4109,7 +4109,7 @@
         <v>4.5819400000000003E-2</v>
       </c>
       <c r="F141">
-        <v>127962</v>
+        <v>127930</v>
       </c>
     </row>
     <row r="142" spans="5:6" x14ac:dyDescent="0.3">
@@ -4117,7 +4117,7 @@
         <v>4.6153800000000002E-2</v>
       </c>
       <c r="F142">
-        <v>127542</v>
+        <v>127509</v>
       </c>
     </row>
     <row r="143" spans="5:6" x14ac:dyDescent="0.3">
@@ -4125,7 +4125,7 @@
         <v>4.6488300000000003E-2</v>
       </c>
       <c r="F143">
-        <v>127125</v>
+        <v>127092</v>
       </c>
     </row>
     <row r="144" spans="5:6" x14ac:dyDescent="0.3">
@@ -4133,7 +4133,7 @@
         <v>4.6822700000000002E-2</v>
       </c>
       <c r="F144">
-        <v>126711</v>
+        <v>126679</v>
       </c>
     </row>
     <row r="145" spans="5:6" x14ac:dyDescent="0.3">
@@ -4141,7 +4141,7 @@
         <v>4.7157200000000003E-2</v>
       </c>
       <c r="F145">
-        <v>126301</v>
+        <v>126268</v>
       </c>
     </row>
     <row r="146" spans="5:6" x14ac:dyDescent="0.3">
@@ -4149,7 +4149,7 @@
         <v>4.7491600000000002E-2</v>
       </c>
       <c r="F146">
-        <v>125894</v>
+        <v>125861</v>
       </c>
     </row>
     <row r="147" spans="5:6" x14ac:dyDescent="0.3">
@@ -4157,7 +4157,7 @@
         <v>4.7826100000000003E-2</v>
       </c>
       <c r="F147">
-        <v>125490</v>
+        <v>125458</v>
       </c>
     </row>
     <row r="148" spans="5:6" x14ac:dyDescent="0.3">
@@ -4165,7 +4165,7 @@
         <v>4.8160500000000002E-2</v>
       </c>
       <c r="F148">
-        <v>125090</v>
+        <v>125058</v>
       </c>
     </row>
     <row r="149" spans="5:6" x14ac:dyDescent="0.3">
@@ -4173,7 +4173,7 @@
         <v>4.8495000000000003E-2</v>
       </c>
       <c r="F149">
-        <v>124693</v>
+        <v>124661</v>
       </c>
     </row>
     <row r="150" spans="5:6" x14ac:dyDescent="0.3">
@@ -4181,7 +4181,7 @@
         <v>4.8829400000000002E-2</v>
       </c>
       <c r="F150">
-        <v>124300</v>
+        <v>124268</v>
       </c>
     </row>
     <row r="151" spans="5:6" x14ac:dyDescent="0.3">
@@ -4189,7 +4189,7 @@
         <v>4.9163900000000003E-2</v>
       </c>
       <c r="F151">
-        <v>123910</v>
+        <v>123879</v>
       </c>
     </row>
     <row r="152" spans="5:6" x14ac:dyDescent="0.3">
@@ -4197,7 +4197,7 @@
         <v>4.9498300000000002E-2</v>
       </c>
       <c r="F152">
-        <v>123524</v>
+        <v>123493</v>
       </c>
     </row>
     <row r="153" spans="5:6" x14ac:dyDescent="0.3">
@@ -4205,7 +4205,7 @@
         <v>4.9832799999999997E-2</v>
       </c>
       <c r="F153">
-        <v>123142</v>
+        <v>123110</v>
       </c>
     </row>
     <row r="154" spans="5:6" x14ac:dyDescent="0.3">
@@ -4213,7 +4213,7 @@
         <v>5.0167200000000002E-2</v>
       </c>
       <c r="F154">
-        <v>122763</v>
+        <v>122731</v>
       </c>
     </row>
     <row r="155" spans="5:6" x14ac:dyDescent="0.3">
@@ -4221,7 +4221,7 @@
         <v>5.0501699999999997E-2</v>
       </c>
       <c r="F155">
-        <v>122387</v>
+        <v>122356</v>
       </c>
     </row>
     <row r="156" spans="5:6" x14ac:dyDescent="0.3">
@@ -4229,7 +4229,7 @@
         <v>5.0836100000000002E-2</v>
       </c>
       <c r="F156">
-        <v>122016</v>
+        <v>121984</v>
       </c>
     </row>
     <row r="157" spans="5:6" x14ac:dyDescent="0.3">
@@ -4237,7 +4237,7 @@
         <v>5.1170599999999997E-2</v>
       </c>
       <c r="F157">
-        <v>121647</v>
+        <v>121616</v>
       </c>
     </row>
     <row r="158" spans="5:6" x14ac:dyDescent="0.3">
@@ -4245,7 +4245,7 @@
         <v>5.1505000000000002E-2</v>
       </c>
       <c r="F158">
-        <v>121283</v>
+        <v>121252</v>
       </c>
     </row>
     <row r="159" spans="5:6" x14ac:dyDescent="0.3">
@@ -4253,7 +4253,7 @@
         <v>5.1839499999999997E-2</v>
       </c>
       <c r="F159">
-        <v>120922</v>
+        <v>120891</v>
       </c>
     </row>
     <row r="160" spans="5:6" x14ac:dyDescent="0.3">
@@ -4261,7 +4261,7 @@
         <v>5.2173900000000002E-2</v>
       </c>
       <c r="F160">
-        <v>120565</v>
+        <v>120534</v>
       </c>
     </row>
     <row r="161" spans="5:6" x14ac:dyDescent="0.3">
@@ -4269,7 +4269,7 @@
         <v>5.2508399999999997E-2</v>
       </c>
       <c r="F161">
-        <v>120212</v>
+        <v>120181</v>
       </c>
     </row>
     <row r="162" spans="5:6" x14ac:dyDescent="0.3">
@@ -4277,7 +4277,7 @@
         <v>5.2842800000000002E-2</v>
       </c>
       <c r="F162">
-        <v>119862</v>
+        <v>119832</v>
       </c>
     </row>
     <row r="163" spans="5:6" x14ac:dyDescent="0.3">
@@ -4285,7 +4285,7 @@
         <v>5.3177299999999997E-2</v>
       </c>
       <c r="F163">
-        <v>119516</v>
+        <v>119486</v>
       </c>
     </row>
     <row r="164" spans="5:6" x14ac:dyDescent="0.3">
@@ -4293,7 +4293,7 @@
         <v>5.3511700000000002E-2</v>
       </c>
       <c r="F164">
-        <v>119174</v>
+        <v>119144</v>
       </c>
     </row>
     <row r="165" spans="5:6" x14ac:dyDescent="0.3">
@@ -4301,7 +4301,7 @@
         <v>5.3846199999999997E-2</v>
       </c>
       <c r="F165">
-        <v>118835</v>
+        <v>118806</v>
       </c>
     </row>
     <row r="166" spans="5:6" x14ac:dyDescent="0.3">
@@ -4309,7 +4309,7 @@
         <v>5.4180600000000002E-2</v>
       </c>
       <c r="F166">
-        <v>118501</v>
+        <v>118471</v>
       </c>
     </row>
     <row r="167" spans="5:6" x14ac:dyDescent="0.3">
@@ -4317,7 +4317,7 @@
         <v>5.4515099999999997E-2</v>
       </c>
       <c r="F167">
-        <v>118170</v>
+        <v>118140</v>
       </c>
     </row>
     <row r="168" spans="5:6" x14ac:dyDescent="0.3">
@@ -4325,7 +4325,7 @@
         <v>5.4849500000000002E-2</v>
       </c>
       <c r="F168">
-        <v>117843</v>
+        <v>117813</v>
       </c>
     </row>
     <row r="169" spans="5:6" x14ac:dyDescent="0.3">
@@ -4333,7 +4333,7 @@
         <v>5.5183900000000001E-2</v>
       </c>
       <c r="F169">
-        <v>117519</v>
+        <v>117490</v>
       </c>
     </row>
     <row r="170" spans="5:6" x14ac:dyDescent="0.3">
@@ -4341,7 +4341,7 @@
         <v>5.5518400000000002E-2</v>
       </c>
       <c r="F170">
-        <v>117200</v>
+        <v>117171</v>
       </c>
     </row>
     <row r="171" spans="5:6" x14ac:dyDescent="0.3">
@@ -4349,7 +4349,7 @@
         <v>5.5852800000000001E-2</v>
       </c>
       <c r="F171">
-        <v>116884</v>
+        <v>116855</v>
       </c>
     </row>
     <row r="172" spans="5:6" x14ac:dyDescent="0.3">
@@ -4357,7 +4357,7 @@
         <v>5.6187300000000003E-2</v>
       </c>
       <c r="F172">
-        <v>116572</v>
+        <v>116543</v>
       </c>
     </row>
     <row r="173" spans="5:6" x14ac:dyDescent="0.3">
@@ -4365,7 +4365,7 @@
         <v>5.6521700000000001E-2</v>
       </c>
       <c r="F173">
-        <v>116263</v>
+        <v>116235</v>
       </c>
     </row>
     <row r="174" spans="5:6" x14ac:dyDescent="0.3">
@@ -4373,7 +4373,7 @@
         <v>5.6856200000000003E-2</v>
       </c>
       <c r="F174">
-        <v>115959</v>
+        <v>115931</v>
       </c>
     </row>
     <row r="175" spans="5:6" x14ac:dyDescent="0.3">
@@ -4381,7 +4381,7 @@
         <v>5.7190600000000001E-2</v>
       </c>
       <c r="F175">
-        <v>115658</v>
+        <v>115630</v>
       </c>
     </row>
     <row r="176" spans="5:6" x14ac:dyDescent="0.3">
@@ -4389,7 +4389,7 @@
         <v>5.7525100000000003E-2</v>
       </c>
       <c r="F176">
-        <v>115361</v>
+        <v>115334</v>
       </c>
     </row>
     <row r="177" spans="5:6" x14ac:dyDescent="0.3">
@@ -4397,7 +4397,7 @@
         <v>5.7859500000000001E-2</v>
       </c>
       <c r="F177">
-        <v>115068</v>
+        <v>115041</v>
       </c>
     </row>
     <row r="178" spans="5:6" x14ac:dyDescent="0.3">
@@ -4405,7 +4405,7 @@
         <v>5.8194000000000003E-2</v>
       </c>
       <c r="F178">
-        <v>114779</v>
+        <v>114752</v>
       </c>
     </row>
     <row r="179" spans="5:6" x14ac:dyDescent="0.3">
@@ -4413,7 +4413,7 @@
         <v>5.8528400000000001E-2</v>
       </c>
       <c r="F179">
-        <v>114493</v>
+        <v>114466</v>
       </c>
     </row>
     <row r="180" spans="5:6" x14ac:dyDescent="0.3">
@@ -4421,7 +4421,7 @@
         <v>5.8862900000000003E-2</v>
       </c>
       <c r="F180">
-        <v>114212</v>
+        <v>114185</v>
       </c>
     </row>
     <row r="181" spans="5:6" x14ac:dyDescent="0.3">
@@ -4429,7 +4429,7 @@
         <v>5.9197300000000001E-2</v>
       </c>
       <c r="F181">
-        <v>113934</v>
+        <v>113907</v>
       </c>
     </row>
     <row r="182" spans="5:6" x14ac:dyDescent="0.3">
@@ -4437,7 +4437,7 @@
         <v>5.9531800000000003E-2</v>
       </c>
       <c r="F182">
-        <v>113659</v>
+        <v>113633</v>
       </c>
     </row>
     <row r="183" spans="5:6" x14ac:dyDescent="0.3">
@@ -4445,7 +4445,7 @@
         <v>5.9866200000000001E-2</v>
       </c>
       <c r="F183">
-        <v>113389</v>
+        <v>113363</v>
       </c>
     </row>
     <row r="184" spans="5:6" x14ac:dyDescent="0.3">
@@ -4453,7 +4453,7 @@
         <v>6.0200700000000003E-2</v>
       </c>
       <c r="F184">
-        <v>113122</v>
+        <v>113096</v>
       </c>
     </row>
     <row r="185" spans="5:6" x14ac:dyDescent="0.3">
@@ -4461,7 +4461,7 @@
         <v>6.0535100000000001E-2</v>
       </c>
       <c r="F185">
-        <v>112859</v>
+        <v>112833</v>
       </c>
     </row>
     <row r="186" spans="5:6" x14ac:dyDescent="0.3">
@@ -4469,7 +4469,7 @@
         <v>6.0869600000000003E-2</v>
       </c>
       <c r="F186">
-        <v>112600</v>
+        <v>112574</v>
       </c>
     </row>
     <row r="187" spans="5:6" x14ac:dyDescent="0.3">
@@ -4477,7 +4477,7 @@
         <v>6.1204000000000001E-2</v>
       </c>
       <c r="F187">
-        <v>112344</v>
+        <v>112319</v>
       </c>
     </row>
     <row r="188" spans="5:6" x14ac:dyDescent="0.3">
@@ -4485,7 +4485,7 @@
         <v>6.1538500000000003E-2</v>
       </c>
       <c r="F188">
-        <v>112092</v>
+        <v>112067</v>
       </c>
     </row>
     <row r="189" spans="5:6" x14ac:dyDescent="0.3">
@@ -4493,7 +4493,7 @@
         <v>6.1872900000000002E-2</v>
       </c>
       <c r="F189">
-        <v>111844</v>
+        <v>111819</v>
       </c>
     </row>
     <row r="190" spans="5:6" x14ac:dyDescent="0.3">
@@ -4501,7 +4501,7 @@
         <v>6.2207400000000003E-2</v>
       </c>
       <c r="F190">
-        <v>111599</v>
+        <v>111575</v>
       </c>
     </row>
     <row r="191" spans="5:6" x14ac:dyDescent="0.3">
@@ -4509,7 +4509,7 @@
         <v>6.2541799999999995E-2</v>
       </c>
       <c r="F191">
-        <v>111358</v>
+        <v>111334</v>
       </c>
     </row>
     <row r="192" spans="5:6" x14ac:dyDescent="0.3">
@@ -4517,7 +4517,7 @@
         <v>6.2876299999999996E-2</v>
       </c>
       <c r="F192">
-        <v>111121</v>
+        <v>111097</v>
       </c>
     </row>
     <row r="193" spans="5:6" x14ac:dyDescent="0.3">
@@ -4525,7 +4525,7 @@
         <v>6.3210699999999995E-2</v>
       </c>
       <c r="F193">
-        <v>110887</v>
+        <v>110863</v>
       </c>
     </row>
     <row r="194" spans="5:6" x14ac:dyDescent="0.3">
@@ -4533,7 +4533,7 @@
         <v>6.3545199999999996E-2</v>
       </c>
       <c r="F194">
-        <v>110657</v>
+        <v>110633</v>
       </c>
     </row>
     <row r="195" spans="5:6" x14ac:dyDescent="0.3">
@@ -4541,7 +4541,7 @@
         <v>6.3879599999999995E-2</v>
       </c>
       <c r="F195">
-        <v>110430</v>
+        <v>110407</v>
       </c>
     </row>
     <row r="196" spans="5:6" x14ac:dyDescent="0.3">
@@ -4549,7 +4549,7 @@
         <v>6.4213999999999993E-2</v>
       </c>
       <c r="F196">
-        <v>110207</v>
+        <v>110184</v>
       </c>
     </row>
     <row r="197" spans="5:6" x14ac:dyDescent="0.3">
@@ -4557,7 +4557,7 @@
         <v>6.4548499999999995E-2</v>
       </c>
       <c r="F197">
-        <v>109987</v>
+        <v>109965</v>
       </c>
     </row>
     <row r="198" spans="5:6" x14ac:dyDescent="0.3">
@@ -4565,7 +4565,7 @@
         <v>6.4882899999999993E-2</v>
       </c>
       <c r="F198">
-        <v>109771</v>
+        <v>109749</v>
       </c>
     </row>
     <row r="199" spans="5:6" x14ac:dyDescent="0.3">
@@ -4573,7 +4573,7 @@
         <v>6.5217399999999995E-2</v>
       </c>
       <c r="F199">
-        <v>109559</v>
+        <v>109536</v>
       </c>
     </row>
     <row r="200" spans="5:6" x14ac:dyDescent="0.3">
@@ -4581,7 +4581,7 @@
         <v>6.5551799999999993E-2</v>
       </c>
       <c r="F200">
-        <v>109350</v>
+        <v>109328</v>
       </c>
     </row>
     <row r="201" spans="5:6" x14ac:dyDescent="0.3">
@@ -4589,7 +4589,7 @@
         <v>6.5886299999999995E-2</v>
       </c>
       <c r="F201">
-        <v>109144</v>
+        <v>109122</v>
       </c>
     </row>
     <row r="202" spans="5:6" x14ac:dyDescent="0.3">
@@ -4597,7 +4597,7 @@
         <v>6.6220699999999993E-2</v>
       </c>
       <c r="F202">
-        <v>108941</v>
+        <v>108920</v>
       </c>
     </row>
     <row r="203" spans="5:6" x14ac:dyDescent="0.3">
@@ -4605,7 +4605,7 @@
         <v>6.6555199999999995E-2</v>
       </c>
       <c r="F203">
-        <v>108743</v>
+        <v>108721</v>
       </c>
     </row>
     <row r="204" spans="5:6" x14ac:dyDescent="0.3">
@@ -4613,7 +4613,7 @@
         <v>6.6889599999999994E-2</v>
       </c>
       <c r="F204">
-        <v>108547</v>
+        <v>108526</v>
       </c>
     </row>
     <row r="205" spans="5:6" x14ac:dyDescent="0.3">
@@ -4621,7 +4621,7 @@
         <v>6.7224099999999995E-2</v>
       </c>
       <c r="F205">
-        <v>108355</v>
+        <v>108334</v>
       </c>
     </row>
     <row r="206" spans="5:6" x14ac:dyDescent="0.3">
@@ -4629,7 +4629,7 @@
         <v>6.7558499999999994E-2</v>
       </c>
       <c r="F206">
-        <v>108166</v>
+        <v>108145</v>
       </c>
     </row>
     <row r="207" spans="5:6" x14ac:dyDescent="0.3">
@@ -4637,7 +4637,7 @@
         <v>6.7892999999999995E-2</v>
       </c>
       <c r="F207">
-        <v>107980</v>
+        <v>107960</v>
       </c>
     </row>
     <row r="208" spans="5:6" x14ac:dyDescent="0.3">
@@ -4645,7 +4645,7 @@
         <v>6.8227399999999994E-2</v>
       </c>
       <c r="F208">
-        <v>107797</v>
+        <v>107778</v>
       </c>
     </row>
     <row r="209" spans="5:6" x14ac:dyDescent="0.3">
@@ -4653,7 +4653,7 @@
         <v>6.8561899999999995E-2</v>
       </c>
       <c r="F209">
-        <v>107618</v>
+        <v>107598</v>
       </c>
     </row>
     <row r="210" spans="5:6" x14ac:dyDescent="0.3">
@@ -4661,7 +4661,7 @@
         <v>6.8896299999999994E-2</v>
       </c>
       <c r="F210">
-        <v>107442</v>
+        <v>107423</v>
       </c>
     </row>
     <row r="211" spans="5:6" x14ac:dyDescent="0.3">
@@ -4669,7 +4669,7 @@
         <v>6.9230799999999995E-2</v>
       </c>
       <c r="F211">
-        <v>107269</v>
+        <v>107250</v>
       </c>
     </row>
     <row r="212" spans="5:6" x14ac:dyDescent="0.3">
@@ -4677,7 +4677,7 @@
         <v>6.9565199999999994E-2</v>
       </c>
       <c r="F212">
-        <v>107099</v>
+        <v>107080</v>
       </c>
     </row>
     <row r="213" spans="5:6" x14ac:dyDescent="0.3">
@@ -4685,7 +4685,7 @@
         <v>6.9899699999999995E-2</v>
       </c>
       <c r="F213">
-        <v>106932</v>
+        <v>106914</v>
       </c>
     </row>
     <row r="214" spans="5:6" x14ac:dyDescent="0.3">
@@ -4693,7 +4693,7 @@
         <v>7.0234099999999994E-2</v>
       </c>
       <c r="F214">
-        <v>106768</v>
+        <v>106750</v>
       </c>
     </row>
     <row r="215" spans="5:6" x14ac:dyDescent="0.3">
@@ -4701,7 +4701,7 @@
         <v>7.0568599999999995E-2</v>
       </c>
       <c r="F215">
-        <v>106607</v>
+        <v>106590</v>
       </c>
     </row>
     <row r="216" spans="5:6" x14ac:dyDescent="0.3">
@@ -4709,7 +4709,7 @@
         <v>7.0902999999999994E-2</v>
       </c>
       <c r="F216">
-        <v>106450</v>
+        <v>106432</v>
       </c>
     </row>
     <row r="217" spans="5:6" x14ac:dyDescent="0.3">
@@ -4717,7 +4717,7 @@
         <v>7.1237499999999995E-2</v>
       </c>
       <c r="F217">
-        <v>106295</v>
+        <v>106277</v>
       </c>
     </row>
     <row r="218" spans="5:6" x14ac:dyDescent="0.3">
@@ -4725,7 +4725,7 @@
         <v>7.1571899999999994E-2</v>
       </c>
       <c r="F218">
-        <v>106143</v>
+        <v>106126</v>
       </c>
     </row>
     <row r="219" spans="5:6" x14ac:dyDescent="0.3">
@@ -4733,7 +4733,7 @@
         <v>7.1906399999999995E-2</v>
       </c>
       <c r="F219">
-        <v>105994</v>
+        <v>105977</v>
       </c>
     </row>
     <row r="220" spans="5:6" x14ac:dyDescent="0.3">
@@ -4741,7 +4741,7 @@
         <v>7.2240799999999994E-2</v>
       </c>
       <c r="F220">
-        <v>105847</v>
+        <v>105831</v>
       </c>
     </row>
     <row r="221" spans="5:6" x14ac:dyDescent="0.3">
@@ -4749,7 +4749,7 @@
         <v>7.2575299999999995E-2</v>
       </c>
       <c r="F221">
-        <v>105704</v>
+        <v>105688</v>
       </c>
     </row>
     <row r="222" spans="5:6" x14ac:dyDescent="0.3">
@@ -4757,7 +4757,7 @@
         <v>7.2909699999999994E-2</v>
       </c>
       <c r="F222">
-        <v>105563</v>
+        <v>105547</v>
       </c>
     </row>
     <row r="223" spans="5:6" x14ac:dyDescent="0.3">
@@ -4765,7 +4765,7 @@
         <v>7.3244100000000006E-2</v>
       </c>
       <c r="F223">
-        <v>105425</v>
+        <v>105409</v>
       </c>
     </row>
     <row r="224" spans="5:6" x14ac:dyDescent="0.3">
@@ -4773,7 +4773,7 @@
         <v>7.3578599999999994E-2</v>
       </c>
       <c r="F224">
-        <v>105290</v>
+        <v>105274</v>
       </c>
     </row>
     <row r="225" spans="5:6" x14ac:dyDescent="0.3">
@@ -4781,7 +4781,7 @@
         <v>7.3913000000000006E-2</v>
       </c>
       <c r="F225">
-        <v>105157</v>
+        <v>105142</v>
       </c>
     </row>
     <row r="226" spans="5:6" x14ac:dyDescent="0.3">
@@ -4789,7 +4789,7 @@
         <v>7.4247499999999994E-2</v>
       </c>
       <c r="F226">
-        <v>105027</v>
+        <v>105012</v>
       </c>
     </row>
     <row r="227" spans="5:6" x14ac:dyDescent="0.3">
@@ -4797,7 +4797,7 @@
         <v>7.4581900000000007E-2</v>
       </c>
       <c r="F227">
-        <v>104900</v>
+        <v>104885</v>
       </c>
     </row>
     <row r="228" spans="5:6" x14ac:dyDescent="0.3">
@@ -4805,7 +4805,7 @@
         <v>7.4916399999999994E-2</v>
       </c>
       <c r="F228">
-        <v>104775</v>
+        <v>104760</v>
       </c>
     </row>
     <row r="229" spans="5:6" x14ac:dyDescent="0.3">
@@ -4813,7 +4813,7 @@
         <v>7.5250800000000007E-2</v>
       </c>
       <c r="F229">
-        <v>104652</v>
+        <v>104638</v>
       </c>
     </row>
     <row r="230" spans="5:6" x14ac:dyDescent="0.3">
@@ -4821,7 +4821,7 @@
         <v>7.5585299999999994E-2</v>
       </c>
       <c r="F230">
-        <v>104533</v>
+        <v>104519</v>
       </c>
     </row>
     <row r="231" spans="5:6" x14ac:dyDescent="0.3">
@@ -4829,7 +4829,7 @@
         <v>7.5919700000000007E-2</v>
       </c>
       <c r="F231">
-        <v>104415</v>
+        <v>104401</v>
       </c>
     </row>
     <row r="232" spans="5:6" x14ac:dyDescent="0.3">
@@ -4837,7 +4837,7 @@
         <v>7.6254199999999994E-2</v>
       </c>
       <c r="F232">
-        <v>104300</v>
+        <v>104287</v>
       </c>
     </row>
     <row r="233" spans="5:6" x14ac:dyDescent="0.3">
@@ -4845,7 +4845,7 @@
         <v>7.6588600000000007E-2</v>
       </c>
       <c r="F233">
-        <v>104187</v>
+        <v>104174</v>
       </c>
     </row>
     <row r="234" spans="5:6" x14ac:dyDescent="0.3">
@@ -4853,7 +4853,7 @@
         <v>7.6923099999999994E-2</v>
       </c>
       <c r="F234">
-        <v>104077</v>
+        <v>104064</v>
       </c>
     </row>
     <row r="235" spans="5:6" x14ac:dyDescent="0.3">
@@ -4861,7 +4861,7 @@
         <v>7.7257500000000007E-2</v>
       </c>
       <c r="F235">
-        <v>103969</v>
+        <v>103956</v>
       </c>
     </row>
     <row r="236" spans="5:6" x14ac:dyDescent="0.3">
@@ -4869,7 +4869,7 @@
         <v>7.7591999999999994E-2</v>
       </c>
       <c r="F236">
-        <v>103863</v>
+        <v>103850</v>
       </c>
     </row>
     <row r="237" spans="5:6" x14ac:dyDescent="0.3">
@@ -4877,7 +4877,7 @@
         <v>7.7926400000000007E-2</v>
       </c>
       <c r="F237">
-        <v>103759</v>
+        <v>103747</v>
       </c>
     </row>
     <row r="238" spans="5:6" x14ac:dyDescent="0.3">
@@ -4885,7 +4885,7 @@
         <v>7.8260899999999994E-2</v>
       </c>
       <c r="F238">
-        <v>103658</v>
+        <v>103646</v>
       </c>
     </row>
     <row r="239" spans="5:6" x14ac:dyDescent="0.3">
@@ -4893,7 +4893,7 @@
         <v>7.8595300000000007E-2</v>
       </c>
       <c r="F239">
-        <v>103558</v>
+        <v>103546</v>
       </c>
     </row>
     <row r="240" spans="5:6" x14ac:dyDescent="0.3">
@@ -4901,7 +4901,7 @@
         <v>7.8929799999999994E-2</v>
       </c>
       <c r="F240">
-        <v>103461</v>
+        <v>103449</v>
       </c>
     </row>
     <row r="241" spans="5:6" x14ac:dyDescent="0.3">
@@ -4909,7 +4909,7 @@
         <v>7.9264200000000007E-2</v>
       </c>
       <c r="F241">
-        <v>103366</v>
+        <v>103354</v>
       </c>
     </row>
     <row r="242" spans="5:6" x14ac:dyDescent="0.3">
@@ -4917,7 +4917,7 @@
         <v>7.9598699999999994E-2</v>
       </c>
       <c r="F242">
-        <v>103272</v>
+        <v>103261</v>
       </c>
     </row>
     <row r="243" spans="5:6" x14ac:dyDescent="0.3">
@@ -4925,7 +4925,7 @@
         <v>7.9933100000000007E-2</v>
       </c>
       <c r="F243">
-        <v>103181</v>
+        <v>103170</v>
       </c>
     </row>
     <row r="244" spans="5:6" x14ac:dyDescent="0.3">
@@ -4933,7 +4933,7 @@
         <v>8.0267599999999995E-2</v>
       </c>
       <c r="F244">
-        <v>103092</v>
+        <v>103081</v>
       </c>
     </row>
     <row r="245" spans="5:6" x14ac:dyDescent="0.3">
@@ -4941,7 +4941,7 @@
         <v>8.0601999999999993E-2</v>
       </c>
       <c r="F245">
-        <v>103004</v>
+        <v>102994</v>
       </c>
     </row>
     <row r="246" spans="5:6" x14ac:dyDescent="0.3">
@@ -4949,7 +4949,7 @@
         <v>8.0936499999999995E-2</v>
       </c>
       <c r="F246">
-        <v>102919</v>
+        <v>102909</v>
       </c>
     </row>
     <row r="247" spans="5:6" x14ac:dyDescent="0.3">
@@ -4957,7 +4957,7 @@
         <v>8.1270899999999993E-2</v>
       </c>
       <c r="F247">
-        <v>102835</v>
+        <v>102825</v>
       </c>
     </row>
     <row r="248" spans="5:6" x14ac:dyDescent="0.3">
@@ -4965,7 +4965,7 @@
         <v>8.1605399999999995E-2</v>
       </c>
       <c r="F248">
-        <v>102753</v>
+        <v>102743</v>
       </c>
     </row>
     <row r="249" spans="5:6" x14ac:dyDescent="0.3">
@@ -4973,7 +4973,7 @@
         <v>8.1939799999999993E-2</v>
       </c>
       <c r="F249">
-        <v>102673</v>
+        <v>102664</v>
       </c>
     </row>
     <row r="250" spans="5:6" x14ac:dyDescent="0.3">
@@ -4981,7 +4981,7 @@
         <v>8.2274200000000006E-2</v>
       </c>
       <c r="F250">
-        <v>102595</v>
+        <v>102585</v>
       </c>
     </row>
     <row r="251" spans="5:6" x14ac:dyDescent="0.3">
@@ -4989,7 +4989,7 @@
         <v>8.2608699999999993E-2</v>
       </c>
       <c r="F251">
-        <v>102518</v>
+        <v>102509</v>
       </c>
     </row>
     <row r="252" spans="5:6" x14ac:dyDescent="0.3">
@@ -4997,7 +4997,7 @@
         <v>8.2943100000000006E-2</v>
       </c>
       <c r="F252">
-        <v>102443</v>
+        <v>102434</v>
       </c>
     </row>
     <row r="253" spans="5:6" x14ac:dyDescent="0.3">
@@ -5005,7 +5005,7 @@
         <v>8.3277599999999993E-2</v>
       </c>
       <c r="F253">
-        <v>102369</v>
+        <v>102361</v>
       </c>
     </row>
     <row r="254" spans="5:6" x14ac:dyDescent="0.3">
@@ -5013,7 +5013,7 @@
         <v>8.3612000000000006E-2</v>
       </c>
       <c r="F254">
-        <v>102297</v>
+        <v>102289</v>
       </c>
     </row>
     <row r="255" spans="5:6" x14ac:dyDescent="0.3">
@@ -5021,7 +5021,7 @@
         <v>8.3946499999999993E-2</v>
       </c>
       <c r="F255">
-        <v>102227</v>
+        <v>102219</v>
       </c>
     </row>
     <row r="256" spans="5:6" x14ac:dyDescent="0.3">
@@ -5029,7 +5029,7 @@
         <v>8.4280900000000006E-2</v>
       </c>
       <c r="F256">
-        <v>102158</v>
+        <v>102150</v>
       </c>
     </row>
     <row r="257" spans="5:6" x14ac:dyDescent="0.3">
@@ -5037,7 +5037,7 @@
         <v>8.4615399999999993E-2</v>
       </c>
       <c r="F257">
-        <v>102091</v>
+        <v>102083</v>
       </c>
     </row>
     <row r="258" spans="5:6" x14ac:dyDescent="0.3">
@@ -5045,7 +5045,7 @@
         <v>8.4949800000000006E-2</v>
       </c>
       <c r="F258">
-        <v>102025</v>
+        <v>102017</v>
       </c>
     </row>
     <row r="259" spans="5:6" x14ac:dyDescent="0.3">
@@ -5053,7 +5053,7 @@
         <v>8.5284299999999993E-2</v>
       </c>
       <c r="F259">
-        <v>101960</v>
+        <v>101953</v>
       </c>
     </row>
     <row r="260" spans="5:6" x14ac:dyDescent="0.3">
@@ -5061,7 +5061,7 @@
         <v>8.5618700000000006E-2</v>
       </c>
       <c r="F260">
-        <v>101897</v>
+        <v>101889</v>
       </c>
     </row>
     <row r="261" spans="5:6" x14ac:dyDescent="0.3">
@@ -5069,7 +5069,7 @@
         <v>8.5953199999999993E-2</v>
       </c>
       <c r="F261">
-        <v>101835</v>
+        <v>101828</v>
       </c>
     </row>
     <row r="262" spans="5:6" x14ac:dyDescent="0.3">
@@ -5077,7 +5077,7 @@
         <v>8.6287600000000006E-2</v>
       </c>
       <c r="F262">
-        <v>101774</v>
+        <v>101767</v>
       </c>
     </row>
     <row r="263" spans="5:6" x14ac:dyDescent="0.3">
@@ -5085,7 +5085,7 @@
         <v>8.6622099999999994E-2</v>
       </c>
       <c r="F263">
-        <v>101715</v>
+        <v>101708</v>
       </c>
     </row>
     <row r="264" spans="5:6" x14ac:dyDescent="0.3">
@@ -5093,7 +5093,7 @@
         <v>8.6956500000000006E-2</v>
       </c>
       <c r="F264">
-        <v>101657</v>
+        <v>101650</v>
       </c>
     </row>
     <row r="265" spans="5:6" x14ac:dyDescent="0.3">
@@ -5101,7 +5101,7 @@
         <v>8.7290999999999994E-2</v>
       </c>
       <c r="F265">
-        <v>101600</v>
+        <v>101593</v>
       </c>
     </row>
     <row r="266" spans="5:6" x14ac:dyDescent="0.3">
@@ -5109,7 +5109,7 @@
         <v>8.7625400000000006E-2</v>
       </c>
       <c r="F266">
-        <v>101544</v>
+        <v>101538</v>
       </c>
     </row>
     <row r="267" spans="5:6" x14ac:dyDescent="0.3">
@@ -5117,7 +5117,7 @@
         <v>8.7959899999999994E-2</v>
       </c>
       <c r="F267">
-        <v>101489</v>
+        <v>101483</v>
       </c>
     </row>
     <row r="268" spans="5:6" x14ac:dyDescent="0.3">
@@ -5125,7 +5125,7 @@
         <v>8.8294300000000006E-2</v>
       </c>
       <c r="F268">
-        <v>101436</v>
+        <v>101430</v>
       </c>
     </row>
     <row r="269" spans="5:6" x14ac:dyDescent="0.3">
@@ -5133,7 +5133,7 @@
         <v>8.8628799999999994E-2</v>
       </c>
       <c r="F269">
-        <v>101383</v>
+        <v>101378</v>
       </c>
     </row>
     <row r="270" spans="5:6" x14ac:dyDescent="0.3">
@@ -5141,7 +5141,7 @@
         <v>8.8963200000000006E-2</v>
       </c>
       <c r="F270">
-        <v>101332</v>
+        <v>101326</v>
       </c>
     </row>
     <row r="271" spans="5:6" x14ac:dyDescent="0.3">
@@ -5149,7 +5149,7 @@
         <v>8.9297699999999994E-2</v>
       </c>
       <c r="F271">
-        <v>101281</v>
+        <v>101276</v>
       </c>
     </row>
     <row r="272" spans="5:6" x14ac:dyDescent="0.3">
@@ -5157,7 +5157,7 @@
         <v>8.9632100000000006E-2</v>
       </c>
       <c r="F272">
-        <v>101231</v>
+        <v>101227</v>
       </c>
     </row>
     <row r="273" spans="5:6" x14ac:dyDescent="0.3">
@@ -5165,7 +5165,7 @@
         <v>8.9966599999999994E-2</v>
       </c>
       <c r="F273">
-        <v>101183</v>
+        <v>101178</v>
       </c>
     </row>
     <row r="274" spans="5:6" x14ac:dyDescent="0.3">
@@ -5173,7 +5173,7 @@
         <v>9.0301000000000006E-2</v>
       </c>
       <c r="F274">
-        <v>101135</v>
+        <v>101131</v>
       </c>
     </row>
     <row r="275" spans="5:6" x14ac:dyDescent="0.3">
@@ -5181,7 +5181,7 @@
         <v>9.0635499999999994E-2</v>
       </c>
       <c r="F275">
-        <v>101088</v>
+        <v>101084</v>
       </c>
     </row>
     <row r="276" spans="5:6" x14ac:dyDescent="0.3">
@@ -5189,7 +5189,7 @@
         <v>9.0969900000000006E-2</v>
       </c>
       <c r="F276">
-        <v>101042</v>
+        <v>101038</v>
       </c>
     </row>
     <row r="277" spans="5:6" x14ac:dyDescent="0.3">
@@ -5197,7 +5197,7 @@
         <v>9.1304300000000005E-2</v>
       </c>
       <c r="F277">
-        <v>100997</v>
+        <v>100993</v>
       </c>
     </row>
     <row r="278" spans="5:6" x14ac:dyDescent="0.3">
@@ -5205,7 +5205,7 @@
         <v>9.1638800000000006E-2</v>
       </c>
       <c r="F278">
-        <v>100952</v>
+        <v>100948</v>
       </c>
     </row>
     <row r="279" spans="5:6" x14ac:dyDescent="0.3">
@@ -5213,7 +5213,7 @@
         <v>9.1973200000000005E-2</v>
       </c>
       <c r="F279">
-        <v>100909</v>
+        <v>100905</v>
       </c>
     </row>
     <row r="280" spans="5:6" x14ac:dyDescent="0.3">
@@ -5221,7 +5221,7 @@
         <v>9.2307700000000006E-2</v>
       </c>
       <c r="F280">
-        <v>100866</v>
+        <v>100862</v>
       </c>
     </row>
     <row r="281" spans="5:6" x14ac:dyDescent="0.3">
@@ -5229,7 +5229,7 @@
         <v>9.2642100000000005E-2</v>
       </c>
       <c r="F281">
-        <v>100823</v>
+        <v>100820</v>
       </c>
     </row>
     <row r="282" spans="5:6" x14ac:dyDescent="0.3">
@@ -5237,7 +5237,7 @@
         <v>9.2976600000000006E-2</v>
       </c>
       <c r="F282">
-        <v>100781</v>
+        <v>100778</v>
       </c>
     </row>
     <row r="283" spans="5:6" x14ac:dyDescent="0.3">
@@ -5245,7 +5245,7 @@
         <v>9.3311000000000005E-2</v>
       </c>
       <c r="F283">
-        <v>100740</v>
+        <v>100737</v>
       </c>
     </row>
     <row r="284" spans="5:6" x14ac:dyDescent="0.3">
@@ -5253,7 +5253,7 @@
         <v>9.3645500000000007E-2</v>
       </c>
       <c r="F284">
-        <v>100700</v>
+        <v>100697</v>
       </c>
     </row>
     <row r="285" spans="5:6" x14ac:dyDescent="0.3">
@@ -5261,7 +5261,7 @@
         <v>9.3979900000000005E-2</v>
       </c>
       <c r="F285">
-        <v>100660</v>
+        <v>100657</v>
       </c>
     </row>
     <row r="286" spans="5:6" x14ac:dyDescent="0.3">
@@ -5269,7 +5269,7 @@
         <v>9.4314400000000007E-2</v>
       </c>
       <c r="F286">
-        <v>100620</v>
+        <v>100618</v>
       </c>
     </row>
     <row r="287" spans="5:6" x14ac:dyDescent="0.3">
@@ -5277,7 +5277,7 @@
         <v>9.4648800000000005E-2</v>
       </c>
       <c r="F287">
-        <v>100581</v>
+        <v>100579</v>
       </c>
     </row>
     <row r="288" spans="5:6" x14ac:dyDescent="0.3">
@@ -5285,7 +5285,7 @@
         <v>9.4983300000000007E-2</v>
       </c>
       <c r="F288">
-        <v>100543</v>
+        <v>100541</v>
       </c>
     </row>
     <row r="289" spans="5:6" x14ac:dyDescent="0.3">
@@ -5293,7 +5293,7 @@
         <v>9.5317700000000005E-2</v>
       </c>
       <c r="F289">
-        <v>100505</v>
+        <v>100503</v>
       </c>
     </row>
     <row r="290" spans="5:6" x14ac:dyDescent="0.3">
@@ -5301,7 +5301,7 @@
         <v>9.5652200000000007E-2</v>
       </c>
       <c r="F290">
-        <v>100467</v>
+        <v>100465</v>
       </c>
     </row>
     <row r="291" spans="5:6" x14ac:dyDescent="0.3">
@@ -5309,7 +5309,7 @@
         <v>9.5986600000000005E-2</v>
       </c>
       <c r="F291">
-        <v>100430</v>
+        <v>100428</v>
       </c>
     </row>
     <row r="292" spans="5:6" x14ac:dyDescent="0.3">
@@ -5317,7 +5317,7 @@
         <v>9.6321100000000007E-2</v>
       </c>
       <c r="F292">
-        <v>100393</v>
+        <v>100391</v>
       </c>
     </row>
     <row r="293" spans="5:6" x14ac:dyDescent="0.3">
@@ -5325,7 +5325,7 @@
         <v>9.6655500000000005E-2</v>
       </c>
       <c r="F293">
-        <v>100356</v>
+        <v>100355</v>
       </c>
     </row>
     <row r="294" spans="5:6" x14ac:dyDescent="0.3">
@@ -5333,7 +5333,7 @@
         <v>9.6990000000000007E-2</v>
       </c>
       <c r="F294">
-        <v>100320</v>
+        <v>100318</v>
       </c>
     </row>
     <row r="295" spans="5:6" x14ac:dyDescent="0.3">
@@ -5341,7 +5341,7 @@
         <v>9.7324400000000005E-2</v>
       </c>
       <c r="F295">
-        <v>100284</v>
+        <v>100282</v>
       </c>
     </row>
     <row r="296" spans="5:6" x14ac:dyDescent="0.3">
@@ -5349,7 +5349,7 @@
         <v>9.7658900000000007E-2</v>
       </c>
       <c r="F296">
-        <v>100248</v>
+        <v>100247</v>
       </c>
     </row>
     <row r="297" spans="5:6" x14ac:dyDescent="0.3">
@@ -5357,7 +5357,7 @@
         <v>9.7993300000000005E-2</v>
       </c>
       <c r="F297">
-        <v>100212</v>
+        <v>100211</v>
       </c>
     </row>
     <row r="298" spans="5:6" x14ac:dyDescent="0.3">
@@ -5373,7 +5373,7 @@
         <v>9.8662200000000005E-2</v>
       </c>
       <c r="F299">
-        <v>100141</v>
+        <v>100140</v>
       </c>
     </row>
     <row r="300" spans="5:6" x14ac:dyDescent="0.3">
@@ -5381,7 +5381,7 @@
         <v>9.8996700000000007E-2</v>
       </c>
       <c r="F300">
-        <v>100106</v>
+        <v>100105</v>
       </c>
     </row>
     <row r="301" spans="5:6" x14ac:dyDescent="0.3">

</xml_diff>